<commit_message>
📊 BIST Screener | 27.05.2026 08:30 | 611 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-27.xlsx
+++ b/data/bist_screener_2026-05-27.xlsx
@@ -25942,34 +25942,38 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>17.67</v>
+        <v>25.7</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0172</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>21980000</v>
-      </c>
-      <c r="E588" s="2" t="inlineStr"/>
+        <v>527150</v>
+      </c>
+      <c r="E588" s="4" t="n">
+        <v>0.9698</v>
+      </c>
       <c r="F588" s="3" t="n">
-        <v>36.71</v>
+        <v>45.64</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
       <c r="I588" s="2" t="inlineStr"/>
-      <c r="J588" s="2" t="inlineStr"/>
+      <c r="J588" s="4" t="n">
+        <v>0.6453</v>
+      </c>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25977,21 +25981,21 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>191.9</v>
+        <v>74.05</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0174</v>
+        <v>-0.0886</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>5800000</v>
+        <v>25520000</v>
       </c>
       <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>55.81</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -25999,7 +26003,7 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
@@ -26012,38 +26016,34 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>25.7</v>
+        <v>191.9</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.006999999999999999</v>
+        <v>-0.0174</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>527150</v>
-      </c>
-      <c r="E590" s="4" t="n">
-        <v>0.9698</v>
-      </c>
+        <v>5800000</v>
+      </c>
+      <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>45.64</v>
+        <v>55.81</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
       <c r="I590" s="2" t="inlineStr"/>
-      <c r="J590" s="4" t="n">
-        <v>0.6453</v>
-      </c>
+      <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26051,21 +26051,21 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>2.6</v>
+        <v>32.18</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>-0.0189</v>
+        <v>0.0255</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>94430000</v>
+        <v>17120000</v>
       </c>
       <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>42.83</v>
+        <v>65.51000000000001</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
@@ -26073,12 +26073,12 @@
       <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26086,147 +26086,149 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>67.15000000000001</v>
+        <v>6.12</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.0121</v>
+        <v>0.009899999999999999</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>562280</v>
-      </c>
-      <c r="E592" s="4" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>8660000</v>
+      </c>
+      <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>54.15</v>
+        <v>54.27</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
       <c r="I592" s="2" t="inlineStr"/>
-      <c r="J592" s="4" t="n">
-        <v>0.1431</v>
-      </c>
+      <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
-        </is>
-      </c>
-      <c r="L592" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr"/>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>70.25</v>
+        <v>129.6</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0.09939999999999999</v>
+        <v>-0.0077</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>42550</v>
+        <v>879570</v>
       </c>
       <c r="E593" s="8" t="n">
-        <v>0.58</v>
+        <v>0.1071</v>
       </c>
       <c r="F593" s="7" t="n">
-        <v>44.2</v>
+        <v>41.79</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="6" t="inlineStr"/>
+      <c r="I593" s="8" t="n">
+        <v>-3.6635</v>
+      </c>
       <c r="J593" s="8" t="n">
-        <v>0.4928</v>
+        <v>-0.4897</v>
       </c>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L593" s="6" t="inlineStr"/>
+          <t>Perakende satış</t>
+        </is>
+      </c>
+      <c r="L593" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+        </is>
+      </c>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>245</v>
+        <v>5.87</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0.0298</v>
+        <v>0.0731</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>9560</v>
+        <v>18100000</v>
       </c>
       <c r="E594" s="4" t="n">
-        <v>0.2578</v>
+        <v>0.1672</v>
       </c>
       <c r="F594" s="3" t="n">
-        <v>50.37</v>
+        <v>49.01</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="2" t="inlineStr"/>
-      <c r="J594" s="2" t="inlineStr"/>
+      <c r="I594" s="4" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J594" s="4" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L594" s="2" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L594" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M594" s="2" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>129.6</v>
+        <v>36.38</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.0077</v>
+        <v>0.0022</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>879570</v>
+        <v>23850000</v>
       </c>
       <c r="E595" s="8" t="n">
-        <v>0.1071</v>
+        <v>0.2667</v>
       </c>
       <c r="F595" s="7" t="n">
-        <v>41.79</v>
+        <v>68.22</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
-      <c r="I595" s="8" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J595" s="8" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I595" s="6" t="inlineStr"/>
+      <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26234,52 +26236,58 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>EKDMR</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>59.85</v>
+        <v>12</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0992</v>
-      </c>
-      <c r="D596" s="2" t="inlineStr"/>
-      <c r="E596" s="2" t="inlineStr"/>
-      <c r="F596" s="2" t="inlineStr"/>
+        <v>0.0345</v>
+      </c>
+      <c r="D596" s="5" t="n">
+        <v>498860</v>
+      </c>
+      <c r="E596" s="4" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F596" s="3" t="n">
+        <v>69.81999999999999</v>
+      </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="2" t="inlineStr"/>
-      <c r="J596" s="2" t="inlineStr"/>
+      <c r="I596" s="4" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J596" s="4" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
-        </is>
-      </c>
-      <c r="L596" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST HALKA ARZ, BIST YILDIZ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L596" s="2" t="inlineStr"/>
       <c r="M596" s="2" t="inlineStr"/>
     </row>
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>13.92</v>
+        <v>2.6</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>-0.0029</v>
+        <v>-0.0189</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>19750000</v>
+        <v>94430000</v>
       </c>
       <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>50.28</v>
+        <v>42.83</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
@@ -26287,12 +26295,12 @@
       <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26300,163 +26308,151 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>39.6</v>
+        <v>70.25</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0365</v>
+        <v>0.09939999999999999</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>11700000</v>
-      </c>
-      <c r="E598" s="2" t="inlineStr"/>
+        <v>42550</v>
+      </c>
+      <c r="E598" s="4" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F598" s="3" t="n">
-        <v>59.52</v>
+        <v>44.2</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
       <c r="I598" s="2" t="inlineStr"/>
-      <c r="J598" s="2" t="inlineStr"/>
+      <c r="J598" s="4" t="n">
+        <v>0.4928</v>
+      </c>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L598" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L598" s="2" t="inlineStr"/>
       <c r="M598" s="2" t="inlineStr"/>
     </row>
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>34.72</v>
+        <v>245</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0012</v>
+        <v>0.0298</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>4640000</v>
+        <v>9560</v>
       </c>
       <c r="E599" s="8" t="n">
-        <v>0.3528</v>
+        <v>0.2578</v>
       </c>
       <c r="F599" s="7" t="n">
-        <v>46.16</v>
-      </c>
-      <c r="G599" s="7" t="n">
-        <v>13.72</v>
-      </c>
+        <v>50.37</v>
+      </c>
+      <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
-      <c r="I599" s="8" t="n">
-        <v>0.1029</v>
-      </c>
-      <c r="J599" s="8" t="n">
-        <v>-1.4864</v>
-      </c>
+      <c r="I599" s="6" t="inlineStr"/>
+      <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
-        </is>
-      </c>
-      <c r="L599" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L599" s="6" t="inlineStr"/>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>36.38</v>
+        <v>80.37</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.0022</v>
+        <v>-0.0042</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>23850000</v>
-      </c>
-      <c r="E600" s="4" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>11050000</v>
+      </c>
+      <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>68.22</v>
+        <v>49.24</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
       <c r="I600" s="2" t="inlineStr"/>
       <c r="J600" s="2" t="inlineStr"/>
-      <c r="K600" s="2" t="inlineStr">
-        <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L600" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+      <c r="K600" s="2" t="inlineStr"/>
+      <c r="L600" s="2" t="inlineStr"/>
       <c r="M600" s="2" t="inlineStr"/>
     </row>
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>80.37</v>
+        <v>13.92</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.0042</v>
+        <v>-0.0029</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>11050000</v>
+        <v>19750000</v>
       </c>
       <c r="E601" s="6" t="inlineStr"/>
       <c r="F601" s="7" t="n">
-        <v>49.24</v>
+        <v>50.28</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
       <c r="I601" s="6" t="inlineStr"/>
       <c r="J601" s="6" t="inlineStr"/>
-      <c r="K601" s="6" t="inlineStr"/>
-      <c r="L601" s="6" t="inlineStr"/>
+      <c r="K601" s="6" t="inlineStr">
+        <is>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L601" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>6.12</v>
+        <v>17.67</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.009899999999999999</v>
+        <v>-0.0172</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>8660000</v>
+        <v>21980000</v>
       </c>
       <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>54.27</v>
+        <v>36.71</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26467,77 +26463,85 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L602" s="2" t="inlineStr"/>
+      <c r="L602" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>12</v>
+        <v>16.49</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0345</v>
+        <v>0.005500000000000001</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>498860</v>
-      </c>
-      <c r="E603" s="8" t="n">
-        <v>0.95</v>
-      </c>
+        <v>28260000</v>
+      </c>
+      <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>69.81999999999999</v>
+        <v>48.12</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="8" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J603" s="8" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I603" s="6" t="inlineStr"/>
+      <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L603" s="6" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L603" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>32.18</v>
+        <v>2.4</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0.0255</v>
+        <v>0</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>17120000</v>
-      </c>
-      <c r="E604" s="2" t="inlineStr"/>
+        <v>16980000</v>
+      </c>
+      <c r="E604" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="F604" s="3" t="n">
-        <v>65.51000000000001</v>
+        <v>39.22</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
-      <c r="I604" s="2" t="inlineStr"/>
-      <c r="J604" s="2" t="inlineStr"/>
+      <c r="I604" s="4" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J604" s="4" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26545,40 +26549,34 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>5.87</v>
+        <v>39.6</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.0731</v>
+        <v>-0.0365</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>18100000</v>
-      </c>
-      <c r="E605" s="8" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>11700000</v>
+      </c>
+      <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>49.01</v>
+        <v>59.52</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
-      <c r="I605" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J605" s="8" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I605" s="6" t="inlineStr"/>
+      <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26586,40 +26584,34 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>2.4</v>
+        <v>16.3</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0</v>
+        <v>-0.0151</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>16980000</v>
-      </c>
-      <c r="E606" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>30420000</v>
+      </c>
+      <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>39.22</v>
+        <v>45.98</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="4" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J606" s="4" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I606" s="2" t="inlineStr"/>
+      <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26627,21 +26619,21 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>16.3</v>
+        <v>77</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.0151</v>
+        <v>0.0158</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>30420000</v>
+        <v>137290</v>
       </c>
       <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>45.98</v>
+        <v>28.48</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26649,47 +26641,47 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L607" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L607" s="6" t="inlineStr"/>
       <c r="M607" s="6" t="inlineStr"/>
     </row>
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>16.49</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>0.005500000000000001</v>
+        <v>0.0121</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>28260000</v>
-      </c>
-      <c r="E608" s="2" t="inlineStr"/>
+        <v>562280</v>
+      </c>
+      <c r="E608" s="4" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F608" s="3" t="n">
-        <v>48.12</v>
+        <v>54.15</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
       <c r="I608" s="2" t="inlineStr"/>
-      <c r="J608" s="2" t="inlineStr"/>
+      <c r="J608" s="4" t="n">
+        <v>0.1431</v>
+      </c>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L608" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M608" s="2" t="inlineStr"/>
@@ -26732,65 +26724,73 @@
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>77</v>
+        <v>34.72</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>0.0158</v>
+        <v>-0.0012</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>137290</v>
-      </c>
-      <c r="E610" s="2" t="inlineStr"/>
+        <v>4640000</v>
+      </c>
+      <c r="E610" s="4" t="n">
+        <v>0.3528</v>
+      </c>
       <c r="F610" s="3" t="n">
-        <v>28.48</v>
-      </c>
-      <c r="G610" s="2" t="inlineStr"/>
+        <v>46.16</v>
+      </c>
+      <c r="G610" s="3" t="n">
+        <v>13.72</v>
+      </c>
       <c r="H610" s="2" t="inlineStr"/>
-      <c r="I610" s="2" t="inlineStr"/>
-      <c r="J610" s="2" t="inlineStr"/>
+      <c r="I610" s="4" t="n">
+        <v>0.1029</v>
+      </c>
+      <c r="J610" s="4" t="n">
+        <v>-1.4864</v>
+      </c>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L610" s="2" t="inlineStr"/>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
+        </is>
+      </c>
+      <c r="L610" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+        </is>
+      </c>
       <c r="M610" s="2" t="inlineStr"/>
     </row>
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>EKDMR</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>170.1</v>
+        <v>59.85</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>-0.023</v>
-      </c>
-      <c r="D611" s="9" t="n">
-        <v>6070000</v>
-      </c>
+        <v>0.0992</v>
+      </c>
+      <c r="D611" s="6" t="inlineStr"/>
       <c r="E611" s="6" t="inlineStr"/>
-      <c r="F611" s="7" t="n">
-        <v>38.2</v>
-      </c>
+      <c r="F611" s="6" t="inlineStr"/>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
       <c r="I611" s="6" t="inlineStr"/>
       <c r="J611" s="6" t="inlineStr"/>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Enerji-dışı mineraller</t>
         </is>
       </c>
       <c r="L611" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST HALKA ARZ, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M611" s="6" t="inlineStr"/>
@@ -26798,21 +26798,21 @@
     <row r="612">
       <c r="A612" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B612" s="3" t="n">
-        <v>74.05</v>
+        <v>170.1</v>
       </c>
       <c r="C612" s="4" t="n">
-        <v>-0.0886</v>
+        <v>-0.023</v>
       </c>
       <c r="D612" s="5" t="n">
-        <v>25520000</v>
+        <v>6070000</v>
       </c>
       <c r="E612" s="2" t="inlineStr"/>
       <c r="F612" s="3" t="n">
-        <v>67.18000000000001</v>
+        <v>38.2</v>
       </c>
       <c r="G612" s="2" t="inlineStr"/>
       <c r="H612" s="2" t="inlineStr"/>
@@ -26820,12 +26820,12 @@
       <c r="J612" s="2" t="inlineStr"/>
       <c r="K612" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L612" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M612" s="2" t="inlineStr"/>
@@ -26852,7 +26852,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>27.05.2026 07:30</t>
+          <t>27.05.2026 08:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 27.05.2026 09:30 | 611 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-27.xlsx
+++ b/data/bist_screener_2026-05-27.xlsx
@@ -25942,38 +25942,34 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>25.7</v>
+        <v>16.49</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.006999999999999999</v>
+        <v>0.005500000000000001</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>527150</v>
-      </c>
-      <c r="E588" s="4" t="n">
-        <v>0.9698</v>
-      </c>
+        <v>28260000</v>
+      </c>
+      <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>45.64</v>
+        <v>48.12</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
       <c r="I588" s="2" t="inlineStr"/>
-      <c r="J588" s="4" t="n">
-        <v>0.6453</v>
-      </c>
+      <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25981,21 +25977,21 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>74.05</v>
+        <v>191.9</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0886</v>
+        <v>-0.0174</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>25520000</v>
+        <v>5800000</v>
       </c>
       <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>67.18000000000001</v>
+        <v>55.81</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -26003,7 +25999,7 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
@@ -26016,21 +26012,21 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>191.9</v>
+        <v>6.12</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.0174</v>
+        <v>0.009899999999999999</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>5800000</v>
+        <v>8660000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>55.81</v>
+        <v>54.27</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
@@ -26038,47 +26034,49 @@
       <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L590" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L590" s="2" t="inlineStr"/>
       <c r="M590" s="2" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>32.18</v>
+        <v>2.4</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0255</v>
+        <v>0</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>17120000</v>
-      </c>
-      <c r="E591" s="6" t="inlineStr"/>
+        <v>16980000</v>
+      </c>
+      <c r="E591" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="F591" s="7" t="n">
-        <v>65.51000000000001</v>
+        <v>39.22</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="6" t="inlineStr"/>
-      <c r="J591" s="6" t="inlineStr"/>
+      <c r="I591" s="8" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J591" s="8" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26086,21 +26084,21 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>6.12</v>
+        <v>77</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.009899999999999999</v>
+        <v>0.0158</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>8660000</v>
+        <v>137290</v>
       </c>
       <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>54.27</v>
+        <v>28.48</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
@@ -26117,81 +26115,77 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>129.6</v>
+        <v>70.25</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0077</v>
+        <v>0.09939999999999999</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>879570</v>
+        <v>42550</v>
       </c>
       <c r="E593" s="8" t="n">
-        <v>0.1071</v>
+        <v>0.58</v>
       </c>
       <c r="F593" s="7" t="n">
-        <v>41.79</v>
+        <v>44.2</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="8" t="n">
-        <v>-3.6635</v>
-      </c>
+      <c r="I593" s="6" t="inlineStr"/>
       <c r="J593" s="8" t="n">
-        <v>-0.4897</v>
+        <v>0.4928</v>
       </c>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
-        </is>
-      </c>
-      <c r="L593" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L593" s="6" t="inlineStr"/>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>5.87</v>
+        <v>34.72</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0.0731</v>
+        <v>-0.0012</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>18100000</v>
+        <v>4640000</v>
       </c>
       <c r="E594" s="4" t="n">
-        <v>0.1672</v>
+        <v>0.3528</v>
       </c>
       <c r="F594" s="3" t="n">
-        <v>49.01</v>
-      </c>
-      <c r="G594" s="2" t="inlineStr"/>
+        <v>46.16</v>
+      </c>
+      <c r="G594" s="3" t="n">
+        <v>13.72</v>
+      </c>
       <c r="H594" s="2" t="inlineStr"/>
       <c r="I594" s="4" t="n">
-        <v>-5.3262</v>
+        <v>0.1029</v>
       </c>
       <c r="J594" s="4" t="n">
-        <v>-4.2562</v>
+        <v>-1.4864</v>
       </c>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26199,108 +26193,96 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>36.38</v>
+        <v>80.37</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.0022</v>
+        <v>-0.0042</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>23850000</v>
-      </c>
-      <c r="E595" s="8" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>11050000</v>
+      </c>
+      <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="7" t="n">
-        <v>68.22</v>
+        <v>49.24</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
       <c r="I595" s="6" t="inlineStr"/>
       <c r="J595" s="6" t="inlineStr"/>
-      <c r="K595" s="6" t="inlineStr">
-        <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L595" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+      <c r="K595" s="6" t="inlineStr"/>
+      <c r="L595" s="6" t="inlineStr"/>
       <c r="M595" s="6" t="inlineStr"/>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>EKDMR</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>12</v>
+        <v>59.85</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0345</v>
-      </c>
-      <c r="D596" s="5" t="n">
-        <v>498860</v>
-      </c>
-      <c r="E596" s="4" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F596" s="3" t="n">
-        <v>69.81999999999999</v>
-      </c>
+        <v>0.0992</v>
+      </c>
+      <c r="D596" s="2" t="inlineStr"/>
+      <c r="E596" s="2" t="inlineStr"/>
+      <c r="F596" s="2" t="inlineStr"/>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="4" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J596" s="4" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I596" s="2" t="inlineStr"/>
+      <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L596" s="2" t="inlineStr"/>
+          <t>Enerji-dışı mineraller</t>
+        </is>
+      </c>
+      <c r="L596" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST HALKA ARZ, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M596" s="2" t="inlineStr"/>
     </row>
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>2.6</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>-0.0189</v>
+        <v>0.0121</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>94430000</v>
-      </c>
-      <c r="E597" s="6" t="inlineStr"/>
+        <v>562280</v>
+      </c>
+      <c r="E597" s="8" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F597" s="7" t="n">
-        <v>42.83</v>
+        <v>54.15</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
       <c r="I597" s="6" t="inlineStr"/>
-      <c r="J597" s="6" t="inlineStr"/>
+      <c r="J597" s="8" t="n">
+        <v>0.1431</v>
+      </c>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26308,58 +26290,56 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>70.25</v>
+        <v>74.05</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>0.09939999999999999</v>
+        <v>-0.0886</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>42550</v>
-      </c>
-      <c r="E598" s="4" t="n">
-        <v>0.58</v>
-      </c>
+        <v>25520000</v>
+      </c>
+      <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>44.2</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
       <c r="I598" s="2" t="inlineStr"/>
-      <c r="J598" s="4" t="n">
-        <v>0.4928</v>
-      </c>
+      <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L598" s="2" t="inlineStr"/>
+          <t>Elektronik teknoloji</t>
+        </is>
+      </c>
+      <c r="L598" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+        </is>
+      </c>
       <c r="M598" s="2" t="inlineStr"/>
     </row>
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>245</v>
+        <v>39.6</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.0298</v>
+        <v>-0.0365</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>9560</v>
-      </c>
-      <c r="E599" s="8" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>11700000</v>
+      </c>
+      <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>50.37</v>
+        <v>59.52</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26367,57 +26347,73 @@
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L599" s="6" t="inlineStr"/>
+          <t>Üretici imalatı</t>
+        </is>
+      </c>
+      <c r="L599" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+        </is>
+      </c>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>80.37</v>
+        <v>25.7</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>-0.0042</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>11050000</v>
-      </c>
-      <c r="E600" s="2" t="inlineStr"/>
+        <v>527150</v>
+      </c>
+      <c r="E600" s="4" t="n">
+        <v>0.9698</v>
+      </c>
       <c r="F600" s="3" t="n">
-        <v>49.24</v>
+        <v>45.64</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
       <c r="I600" s="2" t="inlineStr"/>
-      <c r="J600" s="2" t="inlineStr"/>
-      <c r="K600" s="2" t="inlineStr"/>
-      <c r="L600" s="2" t="inlineStr"/>
+      <c r="J600" s="4" t="n">
+        <v>0.6453</v>
+      </c>
+      <c r="K600" s="2" t="inlineStr">
+        <is>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
+        </is>
+      </c>
+      <c r="L600" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+        </is>
+      </c>
       <c r="M600" s="2" t="inlineStr"/>
     </row>
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>13.92</v>
+        <v>170.1</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.0029</v>
+        <v>-0.023</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>19750000</v>
+        <v>6070000</v>
       </c>
       <c r="E601" s="6" t="inlineStr"/>
       <c r="F601" s="7" t="n">
-        <v>50.28</v>
+        <v>38.2</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
@@ -26425,12 +26421,12 @@
       <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26438,21 +26434,23 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>17.67</v>
+        <v>245</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.0172</v>
+        <v>0.0298</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>21980000</v>
-      </c>
-      <c r="E602" s="2" t="inlineStr"/>
+        <v>9560</v>
+      </c>
+      <c r="E602" s="4" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F602" s="3" t="n">
-        <v>36.71</v>
+        <v>50.37</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26460,88 +26458,80 @@
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L602" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L602" s="2" t="inlineStr"/>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>16.49</v>
+        <v>12</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.005500000000000001</v>
+        <v>0.0345</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>28260000</v>
-      </c>
-      <c r="E603" s="6" t="inlineStr"/>
+        <v>498860</v>
+      </c>
+      <c r="E603" s="8" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F603" s="7" t="n">
-        <v>48.12</v>
+        <v>69.81999999999999</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="6" t="inlineStr"/>
-      <c r="J603" s="6" t="inlineStr"/>
+      <c r="I603" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J603" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L603" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L603" s="6" t="inlineStr"/>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>2.4</v>
+        <v>13.92</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0</v>
+        <v>-0.0029</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>16980000</v>
-      </c>
-      <c r="E604" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>19750000</v>
+      </c>
+      <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>39.22</v>
+        <v>50.28</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
-      <c r="I604" s="4" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J604" s="4" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I604" s="2" t="inlineStr"/>
+      <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26549,21 +26539,21 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>39.6</v>
+        <v>32.18</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.0365</v>
+        <v>0.0255</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>11700000</v>
+        <v>17120000</v>
       </c>
       <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>59.52</v>
+        <v>65.51000000000001</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
@@ -26571,12 +26561,12 @@
       <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26584,34 +26574,40 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>16.3</v>
+        <v>5.87</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.0151</v>
+        <v>0.0731</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>30420000</v>
-      </c>
-      <c r="E606" s="2" t="inlineStr"/>
+        <v>18100000</v>
+      </c>
+      <c r="E606" s="4" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F606" s="3" t="n">
-        <v>45.98</v>
+        <v>49.01</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="2" t="inlineStr"/>
-      <c r="J606" s="2" t="inlineStr"/>
+      <c r="I606" s="4" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J606" s="4" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26619,21 +26615,21 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>77</v>
+        <v>16.3</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>0.0158</v>
+        <v>-0.0151</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>137290</v>
+        <v>30420000</v>
       </c>
       <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>28.48</v>
+        <v>45.98</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26641,47 +26637,47 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L607" s="6" t="inlineStr"/>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L607" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+        </is>
+      </c>
       <c r="M607" s="6" t="inlineStr"/>
     </row>
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>67.15000000000001</v>
+        <v>40.96</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>0.0121</v>
+        <v>0.0039</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>562280</v>
-      </c>
-      <c r="E608" s="4" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>4380000</v>
+      </c>
+      <c r="E608" s="2" t="inlineStr"/>
       <c r="F608" s="3" t="n">
-        <v>54.15</v>
+        <v>50.43</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
       <c r="I608" s="2" t="inlineStr"/>
-      <c r="J608" s="4" t="n">
-        <v>0.1431</v>
-      </c>
+      <c r="J608" s="2" t="inlineStr"/>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L608" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M608" s="2" t="inlineStr"/>
@@ -26689,21 +26685,21 @@
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>40.96</v>
+        <v>2.6</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>0.0039</v>
+        <v>-0.0189</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>4380000</v>
+        <v>94430000</v>
       </c>
       <c r="E609" s="6" t="inlineStr"/>
       <c r="F609" s="7" t="n">
-        <v>50.43</v>
+        <v>42.83</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
@@ -26711,12 +26707,12 @@
       <c r="J609" s="6" t="inlineStr"/>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L609" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M609" s="6" t="inlineStr"/>
@@ -26724,42 +26720,36 @@
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>34.72</v>
+        <v>36.38</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>-0.0012</v>
+        <v>0.0022</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>4640000</v>
+        <v>23850000</v>
       </c>
       <c r="E610" s="4" t="n">
-        <v>0.3528</v>
+        <v>0.2667</v>
       </c>
       <c r="F610" s="3" t="n">
-        <v>46.16</v>
-      </c>
-      <c r="G610" s="3" t="n">
-        <v>13.72</v>
-      </c>
+        <v>68.22</v>
+      </c>
+      <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
-      <c r="I610" s="4" t="n">
-        <v>0.1029</v>
-      </c>
-      <c r="J610" s="4" t="n">
-        <v>-1.4864</v>
-      </c>
+      <c r="I610" s="2" t="inlineStr"/>
+      <c r="J610" s="2" t="inlineStr"/>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L610" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M610" s="2" t="inlineStr"/>
@@ -26767,30 +26757,34 @@
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>EKDMR</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>59.85</v>
+        <v>17.67</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>0.0992</v>
-      </c>
-      <c r="D611" s="6" t="inlineStr"/>
+        <v>-0.0172</v>
+      </c>
+      <c r="D611" s="9" t="n">
+        <v>21980000</v>
+      </c>
       <c r="E611" s="6" t="inlineStr"/>
-      <c r="F611" s="6" t="inlineStr"/>
+      <c r="F611" s="7" t="n">
+        <v>36.71</v>
+      </c>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
       <c r="I611" s="6" t="inlineStr"/>
       <c r="J611" s="6" t="inlineStr"/>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L611" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST HALKA ARZ, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M611" s="6" t="inlineStr"/>
@@ -26798,34 +26792,40 @@
     <row r="612">
       <c r="A612" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B612" s="3" t="n">
-        <v>170.1</v>
+        <v>129.6</v>
       </c>
       <c r="C612" s="4" t="n">
-        <v>-0.023</v>
+        <v>-0.0077</v>
       </c>
       <c r="D612" s="5" t="n">
-        <v>6070000</v>
-      </c>
-      <c r="E612" s="2" t="inlineStr"/>
+        <v>879570</v>
+      </c>
+      <c r="E612" s="4" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F612" s="3" t="n">
-        <v>38.2</v>
+        <v>41.79</v>
       </c>
       <c r="G612" s="2" t="inlineStr"/>
       <c r="H612" s="2" t="inlineStr"/>
-      <c r="I612" s="2" t="inlineStr"/>
-      <c r="J612" s="2" t="inlineStr"/>
+      <c r="I612" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J612" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K612" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L612" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M612" s="2" t="inlineStr"/>
@@ -26852,7 +26852,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>27.05.2026 08:30</t>
+          <t>27.05.2026 09:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 27.05.2026 10:30 | 611 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-27.xlsx
+++ b/data/bist_screener_2026-05-27.xlsx
@@ -25942,21 +25942,21 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>16.49</v>
+        <v>39.6</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.005500000000000001</v>
+        <v>-0.0365</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>28260000</v>
+        <v>11700000</v>
       </c>
       <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>48.12</v>
+        <v>59.52</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
@@ -25964,12 +25964,12 @@
       <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25977,106 +25977,106 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>191.9</v>
+        <v>70.25</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0174</v>
+        <v>0.09939999999999999</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>5800000</v>
-      </c>
-      <c r="E589" s="6" t="inlineStr"/>
+        <v>42550</v>
+      </c>
+      <c r="E589" s="8" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F589" s="7" t="n">
-        <v>55.81</v>
+        <v>44.2</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
       <c r="I589" s="6" t="inlineStr"/>
-      <c r="J589" s="6" t="inlineStr"/>
+      <c r="J589" s="8" t="n">
+        <v>0.4928</v>
+      </c>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L589" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L589" s="6" t="inlineStr"/>
       <c r="M589" s="6" t="inlineStr"/>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>EKDMR</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>6.12</v>
+        <v>59.85</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.009899999999999999</v>
-      </c>
-      <c r="D590" s="5" t="n">
-        <v>8660000</v>
-      </c>
+        <v>0.0992</v>
+      </c>
+      <c r="D590" s="2" t="inlineStr"/>
       <c r="E590" s="2" t="inlineStr"/>
-      <c r="F590" s="3" t="n">
-        <v>54.27</v>
-      </c>
+      <c r="F590" s="2" t="inlineStr"/>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
       <c r="I590" s="2" t="inlineStr"/>
       <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L590" s="2" t="inlineStr"/>
+          <t>Enerji-dışı mineraller</t>
+        </is>
+      </c>
+      <c r="L590" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST HALKA ARZ, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M590" s="2" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>2.4</v>
+        <v>129.6</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0</v>
+        <v>-0.0077</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>16980000</v>
+        <v>879570</v>
       </c>
       <c r="E591" s="8" t="n">
-        <v>1</v>
+        <v>0.1071</v>
       </c>
       <c r="F591" s="7" t="n">
-        <v>39.22</v>
+        <v>41.79</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
       <c r="I591" s="8" t="n">
-        <v>-191.6342</v>
+        <v>-3.6635</v>
       </c>
       <c r="J591" s="8" t="n">
-        <v>-0.8093</v>
+        <v>-0.4897</v>
       </c>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26084,21 +26084,21 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>77</v>
+        <v>13.92</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.0158</v>
+        <v>-0.0029</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>137290</v>
+        <v>19750000</v>
       </c>
       <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>28.48</v>
+        <v>50.28</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
@@ -26106,144 +26106,148 @@
       <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L592" s="2" t="inlineStr"/>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>70.25</v>
+        <v>74.05</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0.09939999999999999</v>
+        <v>-0.0886</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>42550</v>
-      </c>
-      <c r="E593" s="8" t="n">
-        <v>0.58</v>
-      </c>
+        <v>25520000</v>
+      </c>
+      <c r="E593" s="6" t="inlineStr"/>
       <c r="F593" s="7" t="n">
-        <v>44.2</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
       <c r="I593" s="6" t="inlineStr"/>
-      <c r="J593" s="8" t="n">
-        <v>0.4928</v>
-      </c>
+      <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L593" s="6" t="inlineStr"/>
+          <t>Elektronik teknoloji</t>
+        </is>
+      </c>
+      <c r="L593" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+        </is>
+      </c>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>34.72</v>
+        <v>6.12</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.0012</v>
+        <v>0.009899999999999999</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>4640000</v>
-      </c>
-      <c r="E594" s="4" t="n">
-        <v>0.3528</v>
-      </c>
+        <v>8660000</v>
+      </c>
+      <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>46.16</v>
-      </c>
-      <c r="G594" s="3" t="n">
-        <v>13.72</v>
-      </c>
+        <v>54.27</v>
+      </c>
+      <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="4" t="n">
-        <v>0.1029</v>
-      </c>
-      <c r="J594" s="4" t="n">
-        <v>-1.4864</v>
-      </c>
+      <c r="I594" s="2" t="inlineStr"/>
+      <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
-        </is>
-      </c>
-      <c r="L594" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L594" s="2" t="inlineStr"/>
       <c r="M594" s="2" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>80.37</v>
+        <v>170.1</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.0042</v>
+        <v>-0.023</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>11050000</v>
+        <v>6070000</v>
       </c>
       <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="7" t="n">
-        <v>49.24</v>
+        <v>38.2</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
       <c r="I595" s="6" t="inlineStr"/>
       <c r="J595" s="6" t="inlineStr"/>
-      <c r="K595" s="6" t="inlineStr"/>
-      <c r="L595" s="6" t="inlineStr"/>
+      <c r="K595" s="6" t="inlineStr">
+        <is>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L595" s="6" t="inlineStr">
+        <is>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+        </is>
+      </c>
       <c r="M595" s="6" t="inlineStr"/>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>EKDMR</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>59.85</v>
+        <v>40.96</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0992</v>
-      </c>
-      <c r="D596" s="2" t="inlineStr"/>
+        <v>0.0039</v>
+      </c>
+      <c r="D596" s="5" t="n">
+        <v>4380000</v>
+      </c>
       <c r="E596" s="2" t="inlineStr"/>
-      <c r="F596" s="2" t="inlineStr"/>
+      <c r="F596" s="3" t="n">
+        <v>50.43</v>
+      </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
       <c r="I596" s="2" t="inlineStr"/>
       <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST HALKA ARZ, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26251,95 +26255,79 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>67.15000000000001</v>
+        <v>77</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0121</v>
+        <v>0.0158</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>562280</v>
-      </c>
-      <c r="E597" s="8" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>137290</v>
+      </c>
+      <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>54.15</v>
+        <v>28.48</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
       <c r="I597" s="6" t="inlineStr"/>
-      <c r="J597" s="8" t="n">
-        <v>0.1431</v>
-      </c>
+      <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
-        </is>
-      </c>
-      <c r="L597" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L597" s="6" t="inlineStr"/>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>74.05</v>
+        <v>80.37</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0886</v>
+        <v>-0.0042</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>25520000</v>
+        <v>11050000</v>
       </c>
       <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>67.18000000000001</v>
+        <v>49.24</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
       <c r="I598" s="2" t="inlineStr"/>
       <c r="J598" s="2" t="inlineStr"/>
-      <c r="K598" s="2" t="inlineStr">
-        <is>
-          <t>Elektronik teknoloji</t>
-        </is>
-      </c>
-      <c r="L598" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
-        </is>
-      </c>
+      <c r="K598" s="2" t="inlineStr"/>
+      <c r="L598" s="2" t="inlineStr"/>
       <c r="M598" s="2" t="inlineStr"/>
     </row>
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>39.6</v>
+        <v>16.3</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0365</v>
+        <v>-0.0151</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>11700000</v>
+        <v>30420000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>59.52</v>
+        <v>45.98</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26347,12 +26335,12 @@
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26360,38 +26348,40 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>25.7</v>
+        <v>5.87</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>-0.006999999999999999</v>
+        <v>0.0731</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>527150</v>
+        <v>18100000</v>
       </c>
       <c r="E600" s="4" t="n">
-        <v>0.9698</v>
+        <v>0.1672</v>
       </c>
       <c r="F600" s="3" t="n">
-        <v>45.64</v>
+        <v>49.01</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
-      <c r="I600" s="2" t="inlineStr"/>
+      <c r="I600" s="4" t="n">
+        <v>-5.3262</v>
+      </c>
       <c r="J600" s="4" t="n">
-        <v>0.6453</v>
+        <v>-4.2562</v>
       </c>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26399,58 +26389,58 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>170.1</v>
+        <v>12</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.023</v>
+        <v>0.0345</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>6070000</v>
-      </c>
-      <c r="E601" s="6" t="inlineStr"/>
+        <v>498860</v>
+      </c>
+      <c r="E601" s="8" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F601" s="7" t="n">
-        <v>38.2</v>
+        <v>69.81999999999999</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="6" t="inlineStr"/>
-      <c r="J601" s="6" t="inlineStr"/>
+      <c r="I601" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J601" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L601" s="6" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L601" s="6" t="inlineStr"/>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>245</v>
+        <v>2.6</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.0298</v>
+        <v>-0.0189</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>9560</v>
-      </c>
-      <c r="E602" s="4" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>94430000</v>
+      </c>
+      <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>50.37</v>
+        <v>42.83</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26458,67 +26448,75 @@
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L602" s="2" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L602" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>12</v>
+        <v>25.7</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0345</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>498860</v>
+        <v>527150</v>
       </c>
       <c r="E603" s="8" t="n">
-        <v>0.95</v>
+        <v>0.9698</v>
       </c>
       <c r="F603" s="7" t="n">
-        <v>69.81999999999999</v>
+        <v>45.64</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="8" t="n">
-        <v>-23.6291</v>
-      </c>
+      <c r="I603" s="6" t="inlineStr"/>
       <c r="J603" s="8" t="n">
-        <v>-0.4678</v>
+        <v>0.6453</v>
       </c>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L603" s="6" t="inlineStr"/>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
+        </is>
+      </c>
+      <c r="L603" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+        </is>
+      </c>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>13.92</v>
+        <v>36.38</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0029</v>
+        <v>0.0022</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>19750000</v>
-      </c>
-      <c r="E604" s="2" t="inlineStr"/>
+        <v>23850000</v>
+      </c>
+      <c r="E604" s="4" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F604" s="3" t="n">
-        <v>50.28</v>
+        <v>68.22</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26526,12 +26524,12 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26539,21 +26537,21 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>32.18</v>
+        <v>191.9</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.0255</v>
+        <v>-0.0174</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>17120000</v>
+        <v>5800000</v>
       </c>
       <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>65.51000000000001</v>
+        <v>55.81</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
@@ -26561,12 +26559,12 @@
       <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26574,32 +26572,26 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>5.87</v>
+        <v>16.49</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.0731</v>
+        <v>0.005500000000000001</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>18100000</v>
-      </c>
-      <c r="E606" s="4" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>28260000</v>
+      </c>
+      <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>49.01</v>
+        <v>48.12</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="4" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J606" s="4" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I606" s="2" t="inlineStr"/>
+      <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -26607,7 +26599,7 @@
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26615,34 +26607,40 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>16.3</v>
+        <v>2.4</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.0151</v>
+        <v>0</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>30420000</v>
-      </c>
-      <c r="E607" s="6" t="inlineStr"/>
+        <v>16980000</v>
+      </c>
+      <c r="E607" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="F607" s="7" t="n">
-        <v>45.98</v>
+        <v>39.22</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
-      <c r="I607" s="6" t="inlineStr"/>
-      <c r="J607" s="6" t="inlineStr"/>
+      <c r="I607" s="8" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J607" s="8" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26650,21 +26648,23 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>40.96</v>
+        <v>245</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>0.0039</v>
+        <v>0.0298</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>4380000</v>
-      </c>
-      <c r="E608" s="2" t="inlineStr"/>
+        <v>9560</v>
+      </c>
+      <c r="E608" s="4" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F608" s="3" t="n">
-        <v>50.43</v>
+        <v>50.37</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
@@ -26672,47 +26672,47 @@
       <c r="J608" s="2" t="inlineStr"/>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L608" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L608" s="2" t="inlineStr"/>
       <c r="M608" s="2" t="inlineStr"/>
     </row>
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>2.6</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>-0.0189</v>
+        <v>0.0121</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>94430000</v>
-      </c>
-      <c r="E609" s="6" t="inlineStr"/>
+        <v>562280</v>
+      </c>
+      <c r="E609" s="8" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F609" s="7" t="n">
-        <v>42.83</v>
+        <v>54.15</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
       <c r="I609" s="6" t="inlineStr"/>
-      <c r="J609" s="6" t="inlineStr"/>
+      <c r="J609" s="8" t="n">
+        <v>0.1431</v>
+      </c>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L609" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M609" s="6" t="inlineStr"/>
@@ -26720,23 +26720,21 @@
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>36.38</v>
+        <v>32.18</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>0.0022</v>
+        <v>0.0255</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>23850000</v>
-      </c>
-      <c r="E610" s="4" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>17120000</v>
+      </c>
+      <c r="E610" s="2" t="inlineStr"/>
       <c r="F610" s="3" t="n">
-        <v>68.22</v>
+        <v>65.51000000000001</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
@@ -26744,12 +26742,12 @@
       <c r="J610" s="2" t="inlineStr"/>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L610" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M610" s="2" t="inlineStr"/>
@@ -26792,40 +26790,42 @@
     <row r="612">
       <c r="A612" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B612" s="3" t="n">
-        <v>129.6</v>
+        <v>34.72</v>
       </c>
       <c r="C612" s="4" t="n">
-        <v>-0.0077</v>
+        <v>-0.0012</v>
       </c>
       <c r="D612" s="5" t="n">
-        <v>879570</v>
+        <v>4640000</v>
       </c>
       <c r="E612" s="4" t="n">
-        <v>0.1071</v>
+        <v>0.3528</v>
       </c>
       <c r="F612" s="3" t="n">
-        <v>41.79</v>
-      </c>
-      <c r="G612" s="2" t="inlineStr"/>
+        <v>46.16</v>
+      </c>
+      <c r="G612" s="3" t="n">
+        <v>13.72</v>
+      </c>
       <c r="H612" s="2" t="inlineStr"/>
       <c r="I612" s="4" t="n">
-        <v>-3.6635</v>
+        <v>0.1029</v>
       </c>
       <c r="J612" s="4" t="n">
-        <v>-0.4897</v>
+        <v>-1.4864</v>
       </c>
       <c r="K612" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L612" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M612" s="2" t="inlineStr"/>
@@ -26852,7 +26852,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>27.05.2026 09:30</t>
+          <t>27.05.2026 10:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 27.05.2026 11:30 | 611 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-27.xlsx
+++ b/data/bist_screener_2026-05-27.xlsx
@@ -25942,21 +25942,21 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>39.6</v>
+        <v>32.18</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0365</v>
+        <v>0.0255</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>11700000</v>
+        <v>17120000</v>
       </c>
       <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>59.52</v>
+        <v>65.51000000000001</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
@@ -25964,12 +25964,12 @@
       <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25977,36 +25977,36 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>70.25</v>
+        <v>39.6</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>0.09939999999999999</v>
+        <v>-0.0365</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>42550</v>
-      </c>
-      <c r="E589" s="8" t="n">
-        <v>0.58</v>
-      </c>
+        <v>11700000</v>
+      </c>
+      <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>44.2</v>
+        <v>59.52</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
       <c r="I589" s="6" t="inlineStr"/>
-      <c r="J589" s="8" t="n">
-        <v>0.4928</v>
-      </c>
+      <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L589" s="6" t="inlineStr"/>
+          <t>Üretici imalatı</t>
+        </is>
+      </c>
+      <c r="L589" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+        </is>
+      </c>
       <c r="M589" s="6" t="inlineStr"/>
     </row>
     <row r="590">
@@ -26043,40 +26043,34 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>129.6</v>
+        <v>16.3</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>-0.0077</v>
+        <v>-0.0151</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>879570</v>
-      </c>
-      <c r="E591" s="8" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>30420000</v>
+      </c>
+      <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>41.79</v>
+        <v>45.98</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="8" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J591" s="8" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I591" s="6" t="inlineStr"/>
+      <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26084,34 +26078,38 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>13.92</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.0029</v>
+        <v>0.0121</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>19750000</v>
-      </c>
-      <c r="E592" s="2" t="inlineStr"/>
+        <v>562280</v>
+      </c>
+      <c r="E592" s="4" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F592" s="3" t="n">
-        <v>50.28</v>
+        <v>54.15</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
       <c r="I592" s="2" t="inlineStr"/>
-      <c r="J592" s="2" t="inlineStr"/>
+      <c r="J592" s="4" t="n">
+        <v>0.1431</v>
+      </c>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26119,34 +26117,42 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>74.05</v>
+        <v>34.72</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0886</v>
+        <v>-0.0012</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>25520000</v>
-      </c>
-      <c r="E593" s="6" t="inlineStr"/>
+        <v>4640000</v>
+      </c>
+      <c r="E593" s="8" t="n">
+        <v>0.3528</v>
+      </c>
       <c r="F593" s="7" t="n">
-        <v>67.18000000000001</v>
-      </c>
-      <c r="G593" s="6" t="inlineStr"/>
+        <v>46.16</v>
+      </c>
+      <c r="G593" s="7" t="n">
+        <v>13.72</v>
+      </c>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="6" t="inlineStr"/>
-      <c r="J593" s="6" t="inlineStr"/>
+      <c r="I593" s="8" t="n">
+        <v>0.1029</v>
+      </c>
+      <c r="J593" s="8" t="n">
+        <v>-1.4864</v>
+      </c>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26154,52 +26160,62 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>6.12</v>
+        <v>129.6</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0.009899999999999999</v>
+        <v>-0.0077</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>8660000</v>
-      </c>
-      <c r="E594" s="2" t="inlineStr"/>
+        <v>879570</v>
+      </c>
+      <c r="E594" s="4" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F594" s="3" t="n">
-        <v>54.27</v>
+        <v>41.79</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="2" t="inlineStr"/>
-      <c r="J594" s="2" t="inlineStr"/>
+      <c r="I594" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J594" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L594" s="2" t="inlineStr"/>
+          <t>Perakende satış</t>
+        </is>
+      </c>
+      <c r="L594" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+        </is>
+      </c>
       <c r="M594" s="2" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>170.1</v>
+        <v>2.6</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.023</v>
+        <v>-0.0189</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>6070000</v>
+        <v>94430000</v>
       </c>
       <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="7" t="n">
-        <v>38.2</v>
+        <v>42.83</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
@@ -26207,12 +26223,12 @@
       <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26220,34 +26236,38 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>40.96</v>
+        <v>25.7</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0039</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>4380000</v>
-      </c>
-      <c r="E596" s="2" t="inlineStr"/>
+        <v>527150</v>
+      </c>
+      <c r="E596" s="4" t="n">
+        <v>0.9698</v>
+      </c>
       <c r="F596" s="3" t="n">
-        <v>50.43</v>
+        <v>45.64</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
       <c r="I596" s="2" t="inlineStr"/>
-      <c r="J596" s="2" t="inlineStr"/>
+      <c r="J596" s="4" t="n">
+        <v>0.6453</v>
+      </c>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26255,21 +26275,23 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>77</v>
+        <v>36.38</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0158</v>
+        <v>0.0022</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>137290</v>
-      </c>
-      <c r="E597" s="6" t="inlineStr"/>
+        <v>23850000</v>
+      </c>
+      <c r="E597" s="8" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F597" s="7" t="n">
-        <v>28.48</v>
+        <v>68.22</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
@@ -26277,72 +26299,76 @@
       <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L597" s="6" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L597" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>80.37</v>
+        <v>191.9</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0042</v>
+        <v>-0.0174</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>11050000</v>
+        <v>5800000</v>
       </c>
       <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>49.24</v>
+        <v>55.81</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
       <c r="I598" s="2" t="inlineStr"/>
       <c r="J598" s="2" t="inlineStr"/>
-      <c r="K598" s="2" t="inlineStr"/>
-      <c r="L598" s="2" t="inlineStr"/>
+      <c r="K598" s="2" t="inlineStr">
+        <is>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L598" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+        </is>
+      </c>
       <c r="M598" s="2" t="inlineStr"/>
     </row>
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>16.3</v>
+        <v>80.37</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0151</v>
+        <v>-0.0042</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>30420000</v>
+        <v>11050000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>45.98</v>
+        <v>49.24</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
       <c r="I599" s="6" t="inlineStr"/>
       <c r="J599" s="6" t="inlineStr"/>
-      <c r="K599" s="6" t="inlineStr">
-        <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L599" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
-        </is>
-      </c>
+      <c r="K599" s="6" t="inlineStr"/>
+      <c r="L599" s="6" t="inlineStr"/>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
@@ -26389,58 +26415,56 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>12</v>
+        <v>74.05</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.0345</v>
+        <v>-0.0886</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>498860</v>
-      </c>
-      <c r="E601" s="8" t="n">
-        <v>0.95</v>
-      </c>
+        <v>25520000</v>
+      </c>
+      <c r="E601" s="6" t="inlineStr"/>
       <c r="F601" s="7" t="n">
-        <v>69.81999999999999</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="8" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J601" s="8" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I601" s="6" t="inlineStr"/>
+      <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L601" s="6" t="inlineStr"/>
+          <t>Elektronik teknoloji</t>
+        </is>
+      </c>
+      <c r="L601" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+        </is>
+      </c>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>2.6</v>
+        <v>6.12</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.0189</v>
+        <v>0.009899999999999999</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>94430000</v>
+        <v>8660000</v>
       </c>
       <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>42.83</v>
+        <v>54.27</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26451,72 +26475,64 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L602" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+      <c r="L602" s="2" t="inlineStr"/>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>25.7</v>
+        <v>12</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.006999999999999999</v>
+        <v>0.0345</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>527150</v>
+        <v>498860</v>
       </c>
       <c r="E603" s="8" t="n">
-        <v>0.9698</v>
+        <v>0.95</v>
       </c>
       <c r="F603" s="7" t="n">
-        <v>45.64</v>
+        <v>69.81999999999999</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="6" t="inlineStr"/>
+      <c r="I603" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
       <c r="J603" s="8" t="n">
-        <v>0.6453</v>
+        <v>-0.4678</v>
       </c>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
-        </is>
-      </c>
-      <c r="L603" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L603" s="6" t="inlineStr"/>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>36.38</v>
+        <v>40.96</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0.0022</v>
+        <v>0.0039</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>23850000</v>
-      </c>
-      <c r="E604" s="4" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>4380000</v>
+      </c>
+      <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>68.22</v>
+        <v>50.43</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26524,12 +26540,12 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26537,21 +26553,21 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>191.9</v>
+        <v>170.1</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.0174</v>
+        <v>-0.023</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>5800000</v>
+        <v>6070000</v>
       </c>
       <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>55.81</v>
+        <v>38.2</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
@@ -26559,12 +26575,12 @@
       <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26572,21 +26588,21 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>16.49</v>
+        <v>13.92</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.005500000000000001</v>
+        <v>-0.0029</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>28260000</v>
+        <v>19750000</v>
       </c>
       <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>48.12</v>
+        <v>50.28</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
@@ -26594,12 +26610,12 @@
       <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26607,40 +26623,34 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>2.4</v>
+        <v>17.67</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>0</v>
+        <v>-0.0172</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>16980000</v>
-      </c>
-      <c r="E607" s="8" t="n">
-        <v>1</v>
-      </c>
+        <v>21980000</v>
+      </c>
+      <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>39.22</v>
+        <v>36.71</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
-      <c r="I607" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J607" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I607" s="6" t="inlineStr"/>
+      <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26648,23 +26658,21 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>245</v>
+        <v>77</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>0.0298</v>
+        <v>0.0158</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>9560</v>
-      </c>
-      <c r="E608" s="4" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>137290</v>
+      </c>
+      <c r="E608" s="2" t="inlineStr"/>
       <c r="F608" s="3" t="n">
-        <v>50.37</v>
+        <v>28.48</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
@@ -26672,7 +26680,7 @@
       <c r="J608" s="2" t="inlineStr"/>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L608" s="2" t="inlineStr"/>
@@ -26681,38 +26689,34 @@
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>67.15000000000001</v>
+        <v>16.49</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>0.0121</v>
+        <v>0.005500000000000001</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>562280</v>
-      </c>
-      <c r="E609" s="8" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>28260000</v>
+      </c>
+      <c r="E609" s="6" t="inlineStr"/>
       <c r="F609" s="7" t="n">
-        <v>54.15</v>
+        <v>48.12</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
       <c r="I609" s="6" t="inlineStr"/>
-      <c r="J609" s="8" t="n">
-        <v>0.1431</v>
-      </c>
+      <c r="J609" s="6" t="inlineStr"/>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L609" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M609" s="6" t="inlineStr"/>
@@ -26720,21 +26724,23 @@
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>32.18</v>
+        <v>245</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>0.0255</v>
+        <v>0.0298</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>17120000</v>
-      </c>
-      <c r="E610" s="2" t="inlineStr"/>
+        <v>9560</v>
+      </c>
+      <c r="E610" s="4" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F610" s="3" t="n">
-        <v>65.51000000000001</v>
+        <v>50.37</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
@@ -26742,47 +26748,49 @@
       <c r="J610" s="2" t="inlineStr"/>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
-        </is>
-      </c>
-      <c r="L610" s="2" t="inlineStr">
-        <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L610" s="2" t="inlineStr"/>
       <c r="M610" s="2" t="inlineStr"/>
     </row>
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>17.67</v>
+        <v>2.4</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>-0.0172</v>
+        <v>0</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>21980000</v>
-      </c>
-      <c r="E611" s="6" t="inlineStr"/>
+        <v>16980000</v>
+      </c>
+      <c r="E611" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="F611" s="7" t="n">
-        <v>36.71</v>
+        <v>39.22</v>
       </c>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
-      <c r="I611" s="6" t="inlineStr"/>
-      <c r="J611" s="6" t="inlineStr"/>
+      <c r="I611" s="8" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J611" s="8" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L611" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M611" s="6" t="inlineStr"/>
@@ -26790,44 +26798,36 @@
     <row r="612">
       <c r="A612" s="2" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B612" s="3" t="n">
-        <v>34.72</v>
+        <v>70.25</v>
       </c>
       <c r="C612" s="4" t="n">
-        <v>-0.0012</v>
+        <v>0.09939999999999999</v>
       </c>
       <c r="D612" s="5" t="n">
-        <v>4640000</v>
+        <v>42550</v>
       </c>
       <c r="E612" s="4" t="n">
-        <v>0.3528</v>
+        <v>0.58</v>
       </c>
       <c r="F612" s="3" t="n">
-        <v>46.16</v>
-      </c>
-      <c r="G612" s="3" t="n">
-        <v>13.72</v>
-      </c>
+        <v>44.2</v>
+      </c>
+      <c r="G612" s="2" t="inlineStr"/>
       <c r="H612" s="2" t="inlineStr"/>
-      <c r="I612" s="4" t="n">
-        <v>0.1029</v>
-      </c>
+      <c r="I612" s="2" t="inlineStr"/>
       <c r="J612" s="4" t="n">
-        <v>-1.4864</v>
+        <v>0.4928</v>
       </c>
       <c r="K612" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
-        </is>
-      </c>
-      <c r="L612" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L612" s="2" t="inlineStr"/>
       <c r="M612" s="2" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26852,7 +26852,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>27.05.2026 10:30</t>
+          <t>27.05.2026 11:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 27.05.2026 12:30 | 611 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-27.xlsx
+++ b/data/bist_screener_2026-05-27.xlsx
@@ -25942,34 +25942,38 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>32.18</v>
+        <v>25.7</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.0255</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>17120000</v>
-      </c>
-      <c r="E588" s="2" t="inlineStr"/>
+        <v>527150</v>
+      </c>
+      <c r="E588" s="4" t="n">
+        <v>0.9698</v>
+      </c>
       <c r="F588" s="3" t="n">
-        <v>65.51000000000001</v>
+        <v>45.64</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
       <c r="I588" s="2" t="inlineStr"/>
-      <c r="J588" s="2" t="inlineStr"/>
+      <c r="J588" s="4" t="n">
+        <v>0.6453</v>
+      </c>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25977,34 +25981,40 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>39.6</v>
+        <v>5.87</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0365</v>
+        <v>0.0731</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>11700000</v>
-      </c>
-      <c r="E589" s="6" t="inlineStr"/>
+        <v>18100000</v>
+      </c>
+      <c r="E589" s="8" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F589" s="7" t="n">
-        <v>59.52</v>
+        <v>49.01</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
-      <c r="I589" s="6" t="inlineStr"/>
-      <c r="J589" s="6" t="inlineStr"/>
+      <c r="I589" s="8" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J589" s="8" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26012,30 +26022,34 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>EKDMR</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>59.85</v>
+        <v>191.9</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.0992</v>
-      </c>
-      <c r="D590" s="2" t="inlineStr"/>
+        <v>-0.0174</v>
+      </c>
+      <c r="D590" s="5" t="n">
+        <v>5800000</v>
+      </c>
       <c r="E590" s="2" t="inlineStr"/>
-      <c r="F590" s="2" t="inlineStr"/>
+      <c r="F590" s="3" t="n">
+        <v>55.81</v>
+      </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
       <c r="I590" s="2" t="inlineStr"/>
       <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST HALKA ARZ, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26043,21 +26057,23 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>16.3</v>
+        <v>36.38</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>-0.0151</v>
+        <v>0.0022</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>30420000</v>
-      </c>
-      <c r="E591" s="6" t="inlineStr"/>
+        <v>23850000</v>
+      </c>
+      <c r="E591" s="8" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F591" s="7" t="n">
-        <v>45.98</v>
+        <v>68.22</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
@@ -26065,12 +26081,12 @@
       <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26078,38 +26094,34 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>67.15000000000001</v>
+        <v>16.3</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.0121</v>
+        <v>-0.0151</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>562280</v>
-      </c>
-      <c r="E592" s="4" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>30420000</v>
+      </c>
+      <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>54.15</v>
+        <v>45.98</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
       <c r="I592" s="2" t="inlineStr"/>
-      <c r="J592" s="4" t="n">
-        <v>0.1431</v>
-      </c>
+      <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26117,83 +26129,71 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>34.72</v>
+        <v>12</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0012</v>
+        <v>0.0345</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>4640000</v>
+        <v>498860</v>
       </c>
       <c r="E593" s="8" t="n">
-        <v>0.3528</v>
+        <v>0.95</v>
       </c>
       <c r="F593" s="7" t="n">
-        <v>46.16</v>
-      </c>
-      <c r="G593" s="7" t="n">
-        <v>13.72</v>
-      </c>
+        <v>69.81999999999999</v>
+      </c>
+      <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
       <c r="I593" s="8" t="n">
-        <v>0.1029</v>
+        <v>-23.6291</v>
       </c>
       <c r="J593" s="8" t="n">
-        <v>-1.4864</v>
+        <v>-0.4678</v>
       </c>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
-        </is>
-      </c>
-      <c r="L593" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L593" s="6" t="inlineStr"/>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>129.6</v>
+        <v>2.6</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.0077</v>
+        <v>-0.0189</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>879570</v>
-      </c>
-      <c r="E594" s="4" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>94430000</v>
+      </c>
+      <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>41.79</v>
+        <v>42.83</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J594" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I594" s="2" t="inlineStr"/>
+      <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26201,34 +26201,40 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>2.6</v>
+        <v>129.6</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.0189</v>
+        <v>-0.0077</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>94430000</v>
-      </c>
-      <c r="E595" s="6" t="inlineStr"/>
+        <v>879570</v>
+      </c>
+      <c r="E595" s="8" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F595" s="7" t="n">
-        <v>42.83</v>
+        <v>41.79</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
-      <c r="I595" s="6" t="inlineStr"/>
-      <c r="J595" s="6" t="inlineStr"/>
+      <c r="I595" s="8" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J595" s="8" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26236,38 +26242,34 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>25.7</v>
+        <v>13.92</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.006999999999999999</v>
+        <v>-0.0029</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>527150</v>
-      </c>
-      <c r="E596" s="4" t="n">
-        <v>0.9698</v>
-      </c>
+        <v>19750000</v>
+      </c>
+      <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>45.64</v>
+        <v>50.28</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
       <c r="I596" s="2" t="inlineStr"/>
-      <c r="J596" s="4" t="n">
-        <v>0.6453</v>
-      </c>
+      <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26275,23 +26277,21 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>36.38</v>
+        <v>74.05</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0022</v>
+        <v>-0.0886</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>23850000</v>
-      </c>
-      <c r="E597" s="8" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>25520000</v>
+      </c>
+      <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>68.22</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
@@ -26299,12 +26299,12 @@
       <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26312,21 +26312,21 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>191.9</v>
+        <v>17.67</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0174</v>
+        <v>-0.0172</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>5800000</v>
+        <v>21980000</v>
       </c>
       <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>55.81</v>
+        <v>36.71</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
@@ -26334,12 +26334,12 @@
       <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26347,67 +26347,69 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>80.37</v>
+        <v>40.96</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0042</v>
+        <v>0.0039</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>11050000</v>
+        <v>4380000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>49.24</v>
+        <v>50.43</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
       <c r="I599" s="6" t="inlineStr"/>
       <c r="J599" s="6" t="inlineStr"/>
-      <c r="K599" s="6" t="inlineStr"/>
-      <c r="L599" s="6" t="inlineStr"/>
+      <c r="K599" s="6" t="inlineStr">
+        <is>
+          <t>Dayanıklı tüketim malları</t>
+        </is>
+      </c>
+      <c r="L599" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+        </is>
+      </c>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>5.87</v>
+        <v>170.1</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.0731</v>
+        <v>-0.023</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>18100000</v>
-      </c>
-      <c r="E600" s="4" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>6070000</v>
+      </c>
+      <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>49.01</v>
+        <v>38.2</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
-      <c r="I600" s="4" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J600" s="4" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I600" s="2" t="inlineStr"/>
+      <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26415,56 +26417,58 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>74.05</v>
+        <v>70.25</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.0886</v>
+        <v>0.09939999999999999</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>25520000</v>
-      </c>
-      <c r="E601" s="6" t="inlineStr"/>
+        <v>42550</v>
+      </c>
+      <c r="E601" s="8" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F601" s="7" t="n">
-        <v>67.18000000000001</v>
+        <v>44.2</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
       <c r="I601" s="6" t="inlineStr"/>
-      <c r="J601" s="6" t="inlineStr"/>
+      <c r="J601" s="8" t="n">
+        <v>0.4928</v>
+      </c>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
-        </is>
-      </c>
-      <c r="L601" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L601" s="6" t="inlineStr"/>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>6.12</v>
+        <v>245</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.009899999999999999</v>
+        <v>0.0298</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>8660000</v>
-      </c>
-      <c r="E602" s="2" t="inlineStr"/>
+        <v>9560</v>
+      </c>
+      <c r="E602" s="4" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F602" s="3" t="n">
-        <v>54.27</v>
+        <v>50.37</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26472,7 +26476,7 @@
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr"/>
@@ -26481,71 +26485,65 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>12</v>
+        <v>16.49</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0345</v>
+        <v>0.005500000000000001</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>498860</v>
-      </c>
-      <c r="E603" s="8" t="n">
-        <v>0.95</v>
-      </c>
+        <v>28260000</v>
+      </c>
+      <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>69.81999999999999</v>
+        <v>48.12</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="8" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J603" s="8" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I603" s="6" t="inlineStr"/>
+      <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L603" s="6" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L603" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>EKDMR</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>40.96</v>
+        <v>59.85</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0.0039</v>
-      </c>
-      <c r="D604" s="5" t="n">
-        <v>4380000</v>
-      </c>
+        <v>0.0992</v>
+      </c>
+      <c r="D604" s="2" t="inlineStr"/>
       <c r="E604" s="2" t="inlineStr"/>
-      <c r="F604" s="3" t="n">
-        <v>50.43</v>
-      </c>
+      <c r="F604" s="2" t="inlineStr"/>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
       <c r="I604" s="2" t="inlineStr"/>
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Enerji-dışı mineraller</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST HALKA ARZ, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26553,21 +26551,21 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>170.1</v>
+        <v>6.12</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.023</v>
+        <v>0.009899999999999999</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>6070000</v>
+        <v>8660000</v>
       </c>
       <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>38.2</v>
+        <v>54.27</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
@@ -26575,34 +26573,30 @@
       <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L605" s="6" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L605" s="6" t="inlineStr"/>
       <c r="M605" s="6" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>13.92</v>
+        <v>77</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.0029</v>
+        <v>0.0158</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>19750000</v>
+        <v>137290</v>
       </c>
       <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>50.28</v>
+        <v>28.48</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
@@ -26610,34 +26604,30 @@
       <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L606" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L606" s="2" t="inlineStr"/>
       <c r="M606" s="2" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>17.67</v>
+        <v>39.6</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.0172</v>
+        <v>-0.0365</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>21980000</v>
+        <v>11700000</v>
       </c>
       <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>36.71</v>
+        <v>59.52</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26645,12 +26635,12 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26658,52 +26648,62 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>77</v>
+        <v>2.4</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>0.0158</v>
+        <v>0</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>137290</v>
-      </c>
-      <c r="E608" s="2" t="inlineStr"/>
+        <v>16980000</v>
+      </c>
+      <c r="E608" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="F608" s="3" t="n">
-        <v>28.48</v>
+        <v>39.22</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
-      <c r="I608" s="2" t="inlineStr"/>
-      <c r="J608" s="2" t="inlineStr"/>
+      <c r="I608" s="4" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J608" s="4" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L608" s="2" t="inlineStr"/>
+          <t>Dağıtım servisleri</t>
+        </is>
+      </c>
+      <c r="L608" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+        </is>
+      </c>
       <c r="M608" s="2" t="inlineStr"/>
     </row>
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>16.49</v>
+        <v>32.18</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>0.005500000000000001</v>
+        <v>0.0255</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>28260000</v>
+        <v>17120000</v>
       </c>
       <c r="E609" s="6" t="inlineStr"/>
       <c r="F609" s="7" t="n">
-        <v>48.12</v>
+        <v>65.51000000000001</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
@@ -26711,12 +26711,12 @@
       <c r="J609" s="6" t="inlineStr"/>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L609" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M609" s="6" t="inlineStr"/>
@@ -26724,73 +26724,65 @@
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>245</v>
+        <v>80.37</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>0.0298</v>
+        <v>-0.0042</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>9560</v>
-      </c>
-      <c r="E610" s="4" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>11050000</v>
+      </c>
+      <c r="E610" s="2" t="inlineStr"/>
       <c r="F610" s="3" t="n">
-        <v>50.37</v>
+        <v>49.24</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
       <c r="I610" s="2" t="inlineStr"/>
       <c r="J610" s="2" t="inlineStr"/>
-      <c r="K610" s="2" t="inlineStr">
-        <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
+      <c r="K610" s="2" t="inlineStr"/>
       <c r="L610" s="2" t="inlineStr"/>
       <c r="M610" s="2" t="inlineStr"/>
     </row>
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>2.4</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>0</v>
+        <v>0.0121</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>16980000</v>
+        <v>562280</v>
       </c>
       <c r="E611" s="8" t="n">
-        <v>1</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F611" s="7" t="n">
-        <v>39.22</v>
+        <v>54.15</v>
       </c>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
-      <c r="I611" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
+      <c r="I611" s="6" t="inlineStr"/>
       <c r="J611" s="8" t="n">
-        <v>-0.8093</v>
+        <v>0.1431</v>
       </c>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L611" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M611" s="6" t="inlineStr"/>
@@ -26798,36 +26790,44 @@
     <row r="612">
       <c r="A612" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B612" s="3" t="n">
-        <v>70.25</v>
+        <v>34.72</v>
       </c>
       <c r="C612" s="4" t="n">
-        <v>0.09939999999999999</v>
+        <v>-0.0012</v>
       </c>
       <c r="D612" s="5" t="n">
-        <v>42550</v>
+        <v>4640000</v>
       </c>
       <c r="E612" s="4" t="n">
-        <v>0.58</v>
+        <v>0.3528</v>
       </c>
       <c r="F612" s="3" t="n">
-        <v>44.2</v>
-      </c>
-      <c r="G612" s="2" t="inlineStr"/>
+        <v>46.16</v>
+      </c>
+      <c r="G612" s="3" t="n">
+        <v>13.72</v>
+      </c>
       <c r="H612" s="2" t="inlineStr"/>
-      <c r="I612" s="2" t="inlineStr"/>
+      <c r="I612" s="4" t="n">
+        <v>0.1029</v>
+      </c>
       <c r="J612" s="4" t="n">
-        <v>0.4928</v>
+        <v>-1.4864</v>
       </c>
       <c r="K612" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L612" s="2" t="inlineStr"/>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
+        </is>
+      </c>
+      <c r="L612" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+        </is>
+      </c>
       <c r="M612" s="2" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26852,7 +26852,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>27.05.2026 11:30</t>
+          <t>27.05.2026 12:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 27.05.2026 13:30 | 611 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-27.xlsx
+++ b/data/bist_screener_2026-05-27.xlsx
@@ -8708,44 +8708,42 @@
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>BRKSN</t>
+          <t>ERBOS</t>
         </is>
       </c>
       <c r="B190" s="3" t="n">
-        <v>8.539999999999999</v>
+        <v>189.1</v>
       </c>
       <c r="C190" s="4" t="n">
-        <v>0.004699999999999999</v>
+        <v>0.0233</v>
       </c>
       <c r="D190" s="5" t="n">
-        <v>663900</v>
+        <v>88760</v>
       </c>
       <c r="E190" s="4" t="n">
-        <v>0.7524</v>
+        <v>0.7088</v>
       </c>
       <c r="F190" s="3" t="n">
-        <v>43.11</v>
-      </c>
-      <c r="G190" s="3" t="n">
-        <v>32.77</v>
-      </c>
+        <v>43.54</v>
+      </c>
+      <c r="G190" s="2" t="inlineStr"/>
       <c r="H190" s="3" t="n">
         <v>1.01</v>
       </c>
       <c r="I190" s="4" t="n">
-        <v>0.0253</v>
+        <v>-0.0147</v>
       </c>
       <c r="J190" s="4" t="n">
-        <v>2.3941</v>
+        <v>-4.4726</v>
       </c>
       <c r="K190" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Enerji-dışı mineraller</t>
         </is>
       </c>
       <c r="L190" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM TÜM, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST ANA, BIST KAYSERİ</t>
         </is>
       </c>
       <c r="M190" s="2" t="inlineStr"/>
@@ -8753,44 +8751,44 @@
     <row r="191">
       <c r="A191" s="6" t="inlineStr">
         <is>
-          <t>BASGZ</t>
+          <t>BRKSN</t>
         </is>
       </c>
       <c r="B191" s="7" t="n">
-        <v>48.48</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="C191" s="8" t="n">
-        <v>0.009599999999999999</v>
+        <v>0.004699999999999999</v>
       </c>
       <c r="D191" s="9" t="n">
-        <v>364720</v>
+        <v>663900</v>
       </c>
       <c r="E191" s="8" t="n">
-        <v>0.25</v>
+        <v>0.7524</v>
       </c>
       <c r="F191" s="7" t="n">
-        <v>45.52</v>
+        <v>43.11</v>
       </c>
       <c r="G191" s="7" t="n">
-        <v>10.49</v>
+        <v>32.77</v>
       </c>
       <c r="H191" s="7" t="n">
         <v>1.01</v>
       </c>
       <c r="I191" s="8" t="n">
-        <v>0.1117</v>
+        <v>0.0253</v>
       </c>
       <c r="J191" s="8" t="n">
-        <v>3.783</v>
+        <v>2.3941</v>
       </c>
       <c r="K191" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L191" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM TÜM, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M191" s="6" t="inlineStr"/>
@@ -8798,44 +8796,44 @@
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>YKBNK</t>
+          <t>BASGZ</t>
         </is>
       </c>
       <c r="B192" s="3" t="n">
-        <v>33.16</v>
+        <v>48.48</v>
       </c>
       <c r="C192" s="4" t="n">
-        <v>-0.0054</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="D192" s="5" t="n">
-        <v>175060000</v>
+        <v>364720</v>
       </c>
       <c r="E192" s="4" t="n">
-        <v>0.3883</v>
+        <v>0.25</v>
       </c>
       <c r="F192" s="3" t="n">
-        <v>36.28</v>
+        <v>45.52</v>
       </c>
       <c r="G192" s="3" t="n">
-        <v>5</v>
+        <v>10.49</v>
       </c>
       <c r="H192" s="3" t="n">
-        <v>1.03</v>
+        <v>1.01</v>
       </c>
       <c r="I192" s="4" t="n">
-        <v>0.2348</v>
+        <v>0.1117</v>
       </c>
       <c r="J192" s="4" t="n">
-        <v>1.1869</v>
+        <v>3.783</v>
       </c>
       <c r="K192" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L192" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 30, BIST BANKA, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST 50, BIST LİKİT BANKA, BIST MALİ, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST SÜRDÜRÜLEBİLİRLİK 25, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500, STOXX Eastern Europe 50</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M192" s="2" t="inlineStr"/>
@@ -8843,40 +8841,44 @@
     <row r="193">
       <c r="A193" s="6" t="inlineStr">
         <is>
-          <t>KORDS</t>
+          <t>YKBNK</t>
         </is>
       </c>
       <c r="B193" s="7" t="n">
-        <v>85.09999999999999</v>
+        <v>33.16</v>
       </c>
       <c r="C193" s="8" t="n">
-        <v>0.0029</v>
+        <v>-0.0054</v>
       </c>
       <c r="D193" s="9" t="n">
-        <v>4280000</v>
+        <v>175060000</v>
       </c>
       <c r="E193" s="8" t="n">
-        <v>0.2889</v>
+        <v>0.3883</v>
       </c>
       <c r="F193" s="7" t="n">
-        <v>65.81</v>
-      </c>
-      <c r="G193" s="6" t="inlineStr"/>
+        <v>36.28</v>
+      </c>
+      <c r="G193" s="7" t="n">
+        <v>5</v>
+      </c>
       <c r="H193" s="7" t="n">
         <v>1.03</v>
       </c>
       <c r="I193" s="8" t="n">
-        <v>-0.073</v>
-      </c>
-      <c r="J193" s="6" t="inlineStr"/>
+        <v>0.2348</v>
+      </c>
+      <c r="J193" s="8" t="n">
+        <v>1.1869</v>
+      </c>
       <c r="K193" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L193" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TEKSTİL DERİ, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KOCAELI</t>
+          <t>BIST 100, BIST 30, BIST BANKA, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST 50, BIST LİKİT BANKA, BIST MALİ, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST SÜRDÜRÜLEBİLİRLİK 25, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500, STOXX Eastern Europe 50</t>
         </is>
       </c>
       <c r="M193" s="6" t="inlineStr"/>
@@ -8884,44 +8886,40 @@
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>KRGYO</t>
+          <t>KORDS</t>
         </is>
       </c>
       <c r="B194" s="3" t="n">
-        <v>2.72</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="C194" s="4" t="n">
-        <v>0.0037</v>
+        <v>0.0029</v>
       </c>
       <c r="D194" s="5" t="n">
-        <v>6820000</v>
+        <v>4280000</v>
       </c>
       <c r="E194" s="4" t="n">
-        <v>0.3996</v>
+        <v>0.2889</v>
       </c>
       <c r="F194" s="3" t="n">
-        <v>43.79</v>
-      </c>
-      <c r="G194" s="3" t="n">
-        <v>24.07</v>
-      </c>
+        <v>65.81</v>
+      </c>
+      <c r="G194" s="2" t="inlineStr"/>
       <c r="H194" s="3" t="n">
-        <v>1.04</v>
+        <v>1.03</v>
       </c>
       <c r="I194" s="4" t="n">
-        <v>0.0412</v>
-      </c>
-      <c r="J194" s="4" t="n">
-        <v>-5.983300000000001</v>
-      </c>
+        <v>-0.073</v>
+      </c>
+      <c r="J194" s="2" t="inlineStr"/>
       <c r="K194" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L194" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TEKSTİL DERİ, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M194" s="2" t="inlineStr"/>
@@ -8929,42 +8927,44 @@
     <row r="195">
       <c r="A195" s="6" t="inlineStr">
         <is>
-          <t>POLHO</t>
+          <t>KRGYO</t>
         </is>
       </c>
       <c r="B195" s="7" t="n">
-        <v>19.95</v>
+        <v>2.72</v>
       </c>
       <c r="C195" s="8" t="n">
-        <v>-0.0025</v>
+        <v>0.0037</v>
       </c>
       <c r="D195" s="9" t="n">
-        <v>5970000</v>
+        <v>6820000</v>
       </c>
       <c r="E195" s="8" t="n">
-        <v>0.2918</v>
+        <v>0.3996</v>
       </c>
       <c r="F195" s="7" t="n">
-        <v>47.16</v>
-      </c>
-      <c r="G195" s="6" t="inlineStr"/>
+        <v>43.79</v>
+      </c>
+      <c r="G195" s="7" t="n">
+        <v>24.07</v>
+      </c>
       <c r="H195" s="7" t="n">
         <v>1.04</v>
       </c>
       <c r="I195" s="8" t="n">
-        <v>-0.0663</v>
+        <v>0.0412</v>
       </c>
       <c r="J195" s="8" t="n">
-        <v>0.6184000000000001</v>
+        <v>-5.983300000000001</v>
       </c>
       <c r="K195" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L195" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KOCAELI, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M195" s="6" t="inlineStr"/>
@@ -8972,44 +8972,42 @@
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>ULUFA</t>
+          <t>POLHO</t>
         </is>
       </c>
       <c r="B196" s="3" t="n">
-        <v>3.87</v>
+        <v>19.95</v>
       </c>
       <c r="C196" s="4" t="n">
-        <v>0</v>
+        <v>-0.0025</v>
       </c>
       <c r="D196" s="5" t="n">
-        <v>16360000</v>
+        <v>5970000</v>
       </c>
       <c r="E196" s="4" t="n">
-        <v>0.2096</v>
+        <v>0.2918</v>
       </c>
       <c r="F196" s="3" t="n">
-        <v>39.44</v>
-      </c>
-      <c r="G196" s="3" t="n">
-        <v>2.79</v>
-      </c>
+        <v>47.16</v>
+      </c>
+      <c r="G196" s="2" t="inlineStr"/>
       <c r="H196" s="3" t="n">
         <v>1.04</v>
       </c>
       <c r="I196" s="4" t="n">
-        <v>0.3985</v>
+        <v>-0.0663</v>
       </c>
       <c r="J196" s="4" t="n">
-        <v>-0.6119</v>
+        <v>0.6184000000000001</v>
       </c>
       <c r="K196" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L196" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST FIN KIR FAKTÖRIZASYONU, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KOCAELI, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK</t>
         </is>
       </c>
       <c r="M196" s="2" t="inlineStr"/>
@@ -9017,33 +9015,35 @@
     <row r="197">
       <c r="A197" s="6" t="inlineStr">
         <is>
-          <t>SEKFK</t>
+          <t>ULUFA</t>
         </is>
       </c>
       <c r="B197" s="7" t="n">
-        <v>10.27</v>
+        <v>3.87</v>
       </c>
       <c r="C197" s="8" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="D197" s="9" t="n">
-        <v>496110</v>
-      </c>
-      <c r="E197" s="6" t="inlineStr"/>
+        <v>16360000</v>
+      </c>
+      <c r="E197" s="8" t="n">
+        <v>0.2096</v>
+      </c>
       <c r="F197" s="7" t="n">
-        <v>35.39</v>
+        <v>39.44</v>
       </c>
       <c r="G197" s="7" t="n">
-        <v>5.05</v>
+        <v>2.79</v>
       </c>
       <c r="H197" s="7" t="n">
-        <v>1.05</v>
+        <v>1.04</v>
       </c>
       <c r="I197" s="8" t="n">
-        <v>0.2395</v>
+        <v>0.3985</v>
       </c>
       <c r="J197" s="8" t="n">
-        <v>0.4835</v>
+        <v>-0.6119</v>
       </c>
       <c r="K197" s="6" t="inlineStr">
         <is>
@@ -9052,7 +9052,7 @@
       </c>
       <c r="L197" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST FIN KIR FAKTÖRIZASYONU, BIST MALİ, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST FIN KIR FAKTÖRIZASYONU, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M197" s="6" t="inlineStr"/>
@@ -9060,35 +9060,33 @@
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>ISFIN</t>
+          <t>SEKFK</t>
         </is>
       </c>
       <c r="B198" s="3" t="n">
-        <v>19.8</v>
+        <v>10.27</v>
       </c>
       <c r="C198" s="4" t="n">
-        <v>-0.0035</v>
+        <v>0.002</v>
       </c>
       <c r="D198" s="5" t="n">
-        <v>3540000</v>
-      </c>
-      <c r="E198" s="4" t="n">
-        <v>0.4001</v>
-      </c>
+        <v>496110</v>
+      </c>
+      <c r="E198" s="2" t="inlineStr"/>
       <c r="F198" s="3" t="n">
-        <v>46.27</v>
+        <v>35.39</v>
       </c>
       <c r="G198" s="3" t="n">
-        <v>3.62</v>
+        <v>5.05</v>
       </c>
       <c r="H198" s="3" t="n">
-        <v>1.06</v>
+        <v>1.05</v>
       </c>
       <c r="I198" s="4" t="n">
-        <v>0.3434</v>
+        <v>0.2395</v>
       </c>
       <c r="J198" s="4" t="n">
-        <v>-0.273</v>
+        <v>0.4835</v>
       </c>
       <c r="K198" s="2" t="inlineStr">
         <is>
@@ -9097,7 +9095,7 @@
       </c>
       <c r="L198" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST FIN KIR FAKTÖRIZASYONU, BIST MALİ, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST FIN KIR FAKTÖRIZASYONU, BIST MALİ, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M198" s="2" t="inlineStr"/>
@@ -9105,42 +9103,44 @@
     <row r="199">
       <c r="A199" s="6" t="inlineStr">
         <is>
-          <t>BOBET</t>
+          <t>ISFIN</t>
         </is>
       </c>
       <c r="B199" s="7" t="n">
-        <v>18.71</v>
+        <v>19.8</v>
       </c>
       <c r="C199" s="8" t="n">
-        <v>0.0005</v>
+        <v>-0.0035</v>
       </c>
       <c r="D199" s="9" t="n">
-        <v>2910000</v>
+        <v>3540000</v>
       </c>
       <c r="E199" s="8" t="n">
-        <v>0.3</v>
+        <v>0.4001</v>
       </c>
       <c r="F199" s="7" t="n">
-        <v>40.79</v>
-      </c>
-      <c r="G199" s="6" t="inlineStr"/>
+        <v>46.27</v>
+      </c>
+      <c r="G199" s="7" t="n">
+        <v>3.62</v>
+      </c>
       <c r="H199" s="7" t="n">
         <v>1.06</v>
       </c>
       <c r="I199" s="8" t="n">
-        <v>-0.1716</v>
+        <v>0.3434</v>
       </c>
       <c r="J199" s="8" t="n">
-        <v>-2.2777</v>
+        <v>-0.273</v>
       </c>
       <c r="K199" s="6" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L199" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST FIN KIR FAKTÖRIZASYONU, BIST MALİ, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M199" s="6" t="inlineStr"/>
@@ -9148,42 +9148,42 @@
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>IHLAS</t>
+          <t>BOBET</t>
         </is>
       </c>
       <c r="B200" s="3" t="n">
-        <v>2.03</v>
+        <v>18.71</v>
       </c>
       <c r="C200" s="4" t="n">
-        <v>-0.0049</v>
+        <v>0.0005</v>
       </c>
       <c r="D200" s="5" t="n">
-        <v>33600000</v>
+        <v>2910000</v>
       </c>
       <c r="E200" s="4" t="n">
-        <v>0.871</v>
+        <v>0.3</v>
       </c>
       <c r="F200" s="3" t="n">
-        <v>42.85</v>
+        <v>40.79</v>
       </c>
       <c r="G200" s="2" t="inlineStr"/>
       <c r="H200" s="3" t="n">
-        <v>1.07</v>
+        <v>1.06</v>
       </c>
       <c r="I200" s="4" t="n">
-        <v>-0.8428</v>
+        <v>-0.1716</v>
       </c>
       <c r="J200" s="4" t="n">
-        <v>-1.2716</v>
+        <v>-2.2777</v>
       </c>
       <c r="K200" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Enerji-dışı mineraller</t>
         </is>
       </c>
       <c r="L200" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M200" s="2" t="inlineStr"/>
@@ -9191,35 +9191,33 @@
     <row r="201">
       <c r="A201" s="6" t="inlineStr">
         <is>
-          <t>VAKFN</t>
+          <t>IHLAS</t>
         </is>
       </c>
       <c r="B201" s="7" t="n">
-        <v>1.69</v>
+        <v>2.03</v>
       </c>
       <c r="C201" s="8" t="n">
-        <v>-0.0117</v>
-      </c>
-      <c r="D201" s="7" t="n">
-        <v>128140000</v>
+        <v>-0.0049</v>
+      </c>
+      <c r="D201" s="9" t="n">
+        <v>33600000</v>
       </c>
       <c r="E201" s="8" t="n">
-        <v>0.3647</v>
+        <v>0.871</v>
       </c>
       <c r="F201" s="7" t="n">
-        <v>39.78</v>
-      </c>
-      <c r="G201" s="7" t="n">
-        <v>5.03</v>
-      </c>
+        <v>42.85</v>
+      </c>
+      <c r="G201" s="6" t="inlineStr"/>
       <c r="H201" s="7" t="n">
-        <v>1.08</v>
+        <v>1.07</v>
       </c>
       <c r="I201" s="8" t="n">
-        <v>0.2383</v>
+        <v>-0.8428</v>
       </c>
       <c r="J201" s="8" t="n">
-        <v>-0.3663</v>
+        <v>-1.2716</v>
       </c>
       <c r="K201" s="6" t="inlineStr">
         <is>
@@ -9228,7 +9226,7 @@
       </c>
       <c r="L201" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST FIN KIR FAKTÖRIZASYONU, BIST MALİ, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M201" s="6" t="inlineStr"/>
@@ -9236,42 +9234,44 @@
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>ERBOS</t>
+          <t>VAKFN</t>
         </is>
       </c>
       <c r="B202" s="3" t="n">
-        <v>189.1</v>
+        <v>1.69</v>
       </c>
       <c r="C202" s="4" t="n">
-        <v>0.0233</v>
-      </c>
-      <c r="D202" s="5" t="n">
-        <v>88760</v>
+        <v>-0.0117</v>
+      </c>
+      <c r="D202" s="3" t="n">
+        <v>128140000</v>
       </c>
       <c r="E202" s="4" t="n">
-        <v>0.7088</v>
+        <v>0.3647</v>
       </c>
       <c r="F202" s="3" t="n">
-        <v>43.54</v>
-      </c>
-      <c r="G202" s="2" t="inlineStr"/>
+        <v>39.78</v>
+      </c>
+      <c r="G202" s="3" t="n">
+        <v>5.03</v>
+      </c>
       <c r="H202" s="3" t="n">
         <v>1.08</v>
       </c>
       <c r="I202" s="4" t="n">
-        <v>-0.0342</v>
+        <v>0.2383</v>
       </c>
       <c r="J202" s="4" t="n">
-        <v>0.1735</v>
+        <v>-0.3663</v>
       </c>
       <c r="K202" s="2" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L202" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST ANA, BIST KAYSERİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST FIN KIR FAKTÖRIZASYONU, BIST MALİ, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M202" s="2" t="inlineStr"/>
@@ -15592,33 +15592,35 @@
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>HUBVC</t>
+          <t>GARFA</t>
         </is>
       </c>
       <c r="B348" s="3" t="n">
-        <v>3.74</v>
+        <v>29.9</v>
       </c>
       <c r="C348" s="4" t="n">
-        <v>0.1</v>
+        <v>-0.0216</v>
       </c>
       <c r="D348" s="5" t="n">
-        <v>2520000</v>
+        <v>2960000</v>
       </c>
       <c r="E348" s="4" t="n">
-        <v>0.8462000000000001</v>
+        <v>0.08380000000000001</v>
       </c>
       <c r="F348" s="3" t="n">
-        <v>49.84</v>
-      </c>
-      <c r="G348" s="2" t="inlineStr"/>
+        <v>50.06</v>
+      </c>
+      <c r="G348" s="3" t="n">
+        <v>4.95</v>
+      </c>
       <c r="H348" s="3" t="n">
         <v>1.99</v>
       </c>
       <c r="I348" s="4" t="n">
-        <v>-0.9107</v>
+        <v>0.5023</v>
       </c>
       <c r="J348" s="4" t="n">
-        <v>-3.7217</v>
+        <v>0.2491</v>
       </c>
       <c r="K348" s="2" t="inlineStr">
         <is>
@@ -15627,7 +15629,7 @@
       </c>
       <c r="L348" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST MALİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST FIN KIR FAKTÖRIZASYONU, BIST MALİ, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M348" s="2" t="inlineStr"/>
@@ -15635,42 +15637,42 @@
     <row r="349">
       <c r="A349" s="6" t="inlineStr">
         <is>
-          <t>HURGZ</t>
+          <t>HUBVC</t>
         </is>
       </c>
       <c r="B349" s="7" t="n">
-        <v>7.76</v>
+        <v>3.74</v>
       </c>
       <c r="C349" s="8" t="n">
-        <v>-0.0384</v>
+        <v>0.1</v>
       </c>
       <c r="D349" s="9" t="n">
-        <v>20990000</v>
+        <v>2520000</v>
       </c>
       <c r="E349" s="8" t="n">
-        <v>0.1879</v>
+        <v>0.8462000000000001</v>
       </c>
       <c r="F349" s="7" t="n">
-        <v>49.49</v>
+        <v>49.84</v>
       </c>
       <c r="G349" s="6" t="inlineStr"/>
       <c r="H349" s="7" t="n">
-        <v>2.01</v>
+        <v>1.99</v>
       </c>
       <c r="I349" s="8" t="n">
-        <v>-0.4406</v>
+        <v>-0.9107</v>
       </c>
       <c r="J349" s="8" t="n">
-        <v>-11.3341</v>
+        <v>-3.7217</v>
       </c>
       <c r="K349" s="6" t="inlineStr">
         <is>
-          <t>Tüketici hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L349" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST MALİ</t>
         </is>
       </c>
       <c r="M349" s="6" t="inlineStr"/>
@@ -15678,42 +15680,42 @@
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>EKSUN</t>
+          <t>HURGZ</t>
         </is>
       </c>
       <c r="B350" s="3" t="n">
-        <v>7.88</v>
+        <v>7.76</v>
       </c>
       <c r="C350" s="4" t="n">
-        <v>-0.0272</v>
+        <v>-0.0384</v>
       </c>
       <c r="D350" s="5" t="n">
-        <v>18150000</v>
+        <v>20990000</v>
       </c>
       <c r="E350" s="4" t="n">
-        <v>0.2726</v>
+        <v>0.1879</v>
       </c>
       <c r="F350" s="3" t="n">
-        <v>67.93000000000001</v>
+        <v>49.49</v>
       </c>
       <c r="G350" s="2" t="inlineStr"/>
       <c r="H350" s="3" t="n">
-        <v>2.03</v>
+        <v>2.01</v>
       </c>
       <c r="I350" s="4" t="n">
-        <v>-0.1422</v>
+        <v>-0.4406</v>
       </c>
       <c r="J350" s="4" t="n">
-        <v>0.5267000000000001</v>
+        <v>-11.3341</v>
       </c>
       <c r="K350" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Tüketici hizmetleri</t>
         </is>
       </c>
       <c r="L350" s="2" t="inlineStr">
         <is>
-          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M350" s="2" t="inlineStr"/>
@@ -15721,38 +15723,42 @@
     <row r="351">
       <c r="A351" s="6" t="inlineStr">
         <is>
-          <t>FRIGO</t>
+          <t>EKSUN</t>
         </is>
       </c>
       <c r="B351" s="7" t="n">
-        <v>3.17</v>
+        <v>7.88</v>
       </c>
       <c r="C351" s="8" t="n">
-        <v>0.0393</v>
+        <v>-0.0272</v>
       </c>
       <c r="D351" s="9" t="n">
-        <v>40360000</v>
-      </c>
-      <c r="E351" s="6" t="inlineStr"/>
+        <v>18150000</v>
+      </c>
+      <c r="E351" s="8" t="n">
+        <v>0.2726</v>
+      </c>
       <c r="F351" s="7" t="n">
-        <v>51.58</v>
+        <v>67.93000000000001</v>
       </c>
       <c r="G351" s="6" t="inlineStr"/>
       <c r="H351" s="7" t="n">
-        <v>2.04</v>
+        <v>2.03</v>
       </c>
       <c r="I351" s="8" t="n">
-        <v>-0.2194</v>
-      </c>
-      <c r="J351" s="6" t="inlineStr"/>
+        <v>-0.1422</v>
+      </c>
+      <c r="J351" s="8" t="n">
+        <v>0.5267000000000001</v>
+      </c>
       <c r="K351" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L351" s="6" t="inlineStr">
         <is>
-          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST ANA, BIST BURSA</t>
+          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M351" s="6" t="inlineStr"/>
@@ -15760,42 +15766,38 @@
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>HATSN</t>
+          <t>FRIGO</t>
         </is>
       </c>
       <c r="B352" s="3" t="n">
-        <v>58.05</v>
+        <v>3.17</v>
       </c>
       <c r="C352" s="4" t="n">
-        <v>0.09939999999999999</v>
+        <v>0.0393</v>
       </c>
       <c r="D352" s="5" t="n">
-        <v>5610000</v>
-      </c>
-      <c r="E352" s="4" t="n">
-        <v>0.2</v>
-      </c>
+        <v>40360000</v>
+      </c>
+      <c r="E352" s="2" t="inlineStr"/>
       <c r="F352" s="3" t="n">
-        <v>67.64</v>
+        <v>51.58</v>
       </c>
       <c r="G352" s="2" t="inlineStr"/>
       <c r="H352" s="3" t="n">
         <v>2.04</v>
       </c>
       <c r="I352" s="4" t="n">
-        <v>-0.061</v>
-      </c>
-      <c r="J352" s="4" t="n">
-        <v>0.8434999999999999</v>
-      </c>
+        <v>-0.2194</v>
+      </c>
+      <c r="J352" s="2" t="inlineStr"/>
       <c r="K352" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L352" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST ANA, BIST BURSA</t>
         </is>
       </c>
       <c r="M352" s="2" t="inlineStr"/>
@@ -15803,44 +15805,42 @@
     <row r="353">
       <c r="A353" s="6" t="inlineStr">
         <is>
-          <t>ORGE</t>
+          <t>HATSN</t>
         </is>
       </c>
       <c r="B353" s="7" t="n">
-        <v>102</v>
+        <v>58.05</v>
       </c>
       <c r="C353" s="8" t="n">
-        <v>-0.0173</v>
+        <v>0.09939999999999999</v>
       </c>
       <c r="D353" s="9" t="n">
-        <v>3820000</v>
+        <v>5610000</v>
       </c>
       <c r="E353" s="8" t="n">
-        <v>0.4719</v>
+        <v>0.2</v>
       </c>
       <c r="F353" s="7" t="n">
-        <v>63.98</v>
-      </c>
-      <c r="G353" s="7" t="n">
-        <v>14.1</v>
-      </c>
+        <v>67.64</v>
+      </c>
+      <c r="G353" s="6" t="inlineStr"/>
       <c r="H353" s="7" t="n">
         <v>2.04</v>
       </c>
       <c r="I353" s="8" t="n">
-        <v>0.1767</v>
+        <v>-0.061</v>
       </c>
       <c r="J353" s="8" t="n">
-        <v>0.8362999999999999</v>
+        <v>0.8434999999999999</v>
       </c>
       <c r="K353" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L353" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M353" s="6" t="inlineStr"/>
@@ -15848,42 +15848,44 @@
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>OBAMS</t>
+          <t>ORGE</t>
         </is>
       </c>
       <c r="B354" s="3" t="n">
-        <v>7.96</v>
+        <v>102</v>
       </c>
       <c r="C354" s="4" t="n">
-        <v>-0.0221</v>
+        <v>-0.0173</v>
       </c>
       <c r="D354" s="5" t="n">
-        <v>82570000</v>
+        <v>3820000</v>
       </c>
       <c r="E354" s="4" t="n">
-        <v>0.2611</v>
+        <v>0.4719</v>
       </c>
       <c r="F354" s="3" t="n">
-        <v>38.53</v>
-      </c>
-      <c r="G354" s="2" t="inlineStr"/>
+        <v>63.98</v>
+      </c>
+      <c r="G354" s="3" t="n">
+        <v>14.1</v>
+      </c>
       <c r="H354" s="3" t="n">
         <v>2.04</v>
       </c>
       <c r="I354" s="4" t="n">
-        <v>-0.2839</v>
+        <v>0.1767</v>
       </c>
       <c r="J354" s="4" t="n">
-        <v>0.0165</v>
+        <v>0.8362999999999999</v>
       </c>
       <c r="K354" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L354" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M354" s="2" t="inlineStr"/>
@@ -15891,35 +15893,33 @@
     <row r="355">
       <c r="A355" s="6" t="inlineStr">
         <is>
-          <t>SUNTK</t>
+          <t>OBAMS</t>
         </is>
       </c>
       <c r="B355" s="7" t="n">
-        <v>33.24</v>
+        <v>7.96</v>
       </c>
       <c r="C355" s="8" t="n">
-        <v>0.0342</v>
+        <v>-0.0221</v>
       </c>
       <c r="D355" s="9" t="n">
-        <v>1190000</v>
+        <v>82570000</v>
       </c>
       <c r="E355" s="8" t="n">
-        <v>0.2071</v>
+        <v>0.2611</v>
       </c>
       <c r="F355" s="7" t="n">
-        <v>42.66</v>
-      </c>
-      <c r="G355" s="7" t="n">
-        <v>26.8</v>
-      </c>
+        <v>38.53</v>
+      </c>
+      <c r="G355" s="6" t="inlineStr"/>
       <c r="H355" s="7" t="n">
-        <v>2.05</v>
+        <v>2.04</v>
       </c>
       <c r="I355" s="8" t="n">
-        <v>0.0868</v>
+        <v>-0.2839</v>
       </c>
       <c r="J355" s="8" t="n">
-        <v>-1.3585</v>
+        <v>0.0165</v>
       </c>
       <c r="K355" s="6" t="inlineStr">
         <is>
@@ -15928,7 +15928,7 @@
       </c>
       <c r="L355" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TEKSTİL DERİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KATILIM TEMETTU, BIST İZMİR, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M355" s="6" t="inlineStr"/>
@@ -15936,44 +15936,44 @@
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>OFSYM</t>
+          <t>SUNTK</t>
         </is>
       </c>
       <c r="B356" s="3" t="n">
-        <v>58.35</v>
+        <v>33.24</v>
       </c>
       <c r="C356" s="4" t="n">
-        <v>-0.016</v>
+        <v>0.0342</v>
       </c>
       <c r="D356" s="5" t="n">
         <v>1190000</v>
       </c>
       <c r="E356" s="4" t="n">
-        <v>0.1556</v>
+        <v>0.2071</v>
       </c>
       <c r="F356" s="3" t="n">
-        <v>46.99</v>
+        <v>42.66</v>
       </c>
       <c r="G356" s="3" t="n">
-        <v>28.97</v>
+        <v>26.8</v>
       </c>
       <c r="H356" s="3" t="n">
-        <v>2.07</v>
+        <v>2.05</v>
       </c>
       <c r="I356" s="4" t="n">
-        <v>0.08449999999999999</v>
+        <v>0.0868</v>
       </c>
       <c r="J356" s="4" t="n">
-        <v>0.1882</v>
+        <v>-1.3585</v>
       </c>
       <c r="K356" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L356" s="2" t="inlineStr">
         <is>
-          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST ANA, BIST ANKARA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TEKSTİL DERİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KATILIM TEMETTU, BIST İZMİR, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK</t>
         </is>
       </c>
       <c r="M356" s="2" t="inlineStr"/>
@@ -15981,42 +15981,44 @@
     <row r="357">
       <c r="A357" s="6" t="inlineStr">
         <is>
-          <t>EGEEN</t>
-        </is>
-      </c>
-      <c r="B357" s="9" t="n">
-        <v>5635</v>
+          <t>OFSYM</t>
+        </is>
+      </c>
+      <c r="B357" s="7" t="n">
+        <v>58.35</v>
       </c>
       <c r="C357" s="8" t="n">
-        <v>-0.0114</v>
+        <v>-0.016</v>
       </c>
       <c r="D357" s="9" t="n">
-        <v>13790</v>
+        <v>1190000</v>
       </c>
       <c r="E357" s="8" t="n">
-        <v>0.3637</v>
+        <v>0.1556</v>
       </c>
       <c r="F357" s="7" t="n">
-        <v>38.87</v>
-      </c>
-      <c r="G357" s="6" t="inlineStr"/>
+        <v>46.99</v>
+      </c>
+      <c r="G357" s="7" t="n">
+        <v>28.97</v>
+      </c>
       <c r="H357" s="7" t="n">
-        <v>2.1</v>
+        <v>2.07</v>
       </c>
       <c r="I357" s="8" t="n">
-        <v>-0.0341</v>
+        <v>0.08449999999999999</v>
       </c>
       <c r="J357" s="8" t="n">
-        <v>0.3126</v>
+        <v>0.1882</v>
       </c>
       <c r="K357" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L357" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST YILDIZ, BIST İZMİR</t>
+          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST ANA, BIST ANKARA</t>
         </is>
       </c>
       <c r="M357" s="6" t="inlineStr"/>
@@ -16024,40 +16026,42 @@
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>AKHAN</t>
-        </is>
-      </c>
-      <c r="B358" s="3" t="n">
-        <v>29.24</v>
+          <t>EGEEN</t>
+        </is>
+      </c>
+      <c r="B358" s="5" t="n">
+        <v>5635</v>
       </c>
       <c r="C358" s="4" t="n">
-        <v>-0.0102</v>
+        <v>-0.0114</v>
       </c>
       <c r="D358" s="5" t="n">
-        <v>6160000</v>
+        <v>13790</v>
       </c>
       <c r="E358" s="4" t="n">
-        <v>0.2001</v>
+        <v>0.3637</v>
       </c>
       <c r="F358" s="3" t="n">
-        <v>56.05</v>
+        <v>38.87</v>
       </c>
       <c r="G358" s="2" t="inlineStr"/>
       <c r="H358" s="3" t="n">
-        <v>2.14</v>
+        <v>2.1</v>
       </c>
       <c r="I358" s="4" t="n">
-        <v>0.0438</v>
-      </c>
-      <c r="J358" s="2" t="inlineStr"/>
+        <v>-0.0341</v>
+      </c>
+      <c r="J358" s="4" t="n">
+        <v>0.3126</v>
+      </c>
       <c r="K358" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L358" s="2" t="inlineStr">
         <is>
-          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST YILDIZ, BIST İZMİR</t>
         </is>
       </c>
       <c r="M358" s="2" t="inlineStr"/>
@@ -16065,44 +16069,40 @@
     <row r="359">
       <c r="A359" s="6" t="inlineStr">
         <is>
-          <t>BEYAZ</t>
+          <t>AKHAN</t>
         </is>
       </c>
       <c r="B359" s="7" t="n">
-        <v>28.76</v>
+        <v>29.24</v>
       </c>
       <c r="C359" s="8" t="n">
-        <v>0.0113</v>
+        <v>-0.0102</v>
       </c>
       <c r="D359" s="9" t="n">
-        <v>812270</v>
+        <v>6160000</v>
       </c>
       <c r="E359" s="8" t="n">
-        <v>0.2455</v>
+        <v>0.2001</v>
       </c>
       <c r="F359" s="7" t="n">
-        <v>46.76</v>
-      </c>
-      <c r="G359" s="7" t="n">
-        <v>22.5</v>
-      </c>
+        <v>56.05</v>
+      </c>
+      <c r="G359" s="6" t="inlineStr"/>
       <c r="H359" s="7" t="n">
-        <v>2.15</v>
+        <v>2.14</v>
       </c>
       <c r="I359" s="8" t="n">
-        <v>0.1128</v>
-      </c>
-      <c r="J359" s="8" t="n">
-        <v>-0.9066</v>
-      </c>
+        <v>0.0438</v>
+      </c>
+      <c r="J359" s="6" t="inlineStr"/>
       <c r="K359" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L359" s="6" t="inlineStr">
         <is>
-          <t>BIST ULASTIRMA, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST ANA, BIST BALIKESİR</t>
+          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M359" s="6" t="inlineStr"/>
@@ -16110,42 +16110,44 @@
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>ERSU</t>
+          <t>BEYAZ</t>
         </is>
       </c>
       <c r="B360" s="3" t="n">
-        <v>25.5</v>
+        <v>28.76</v>
       </c>
       <c r="C360" s="4" t="n">
-        <v>-0.0016</v>
+        <v>0.0113</v>
       </c>
       <c r="D360" s="5" t="n">
-        <v>542670</v>
+        <v>812270</v>
       </c>
       <c r="E360" s="4" t="n">
-        <v>0.7902</v>
+        <v>0.2455</v>
       </c>
       <c r="F360" s="3" t="n">
-        <v>47.64</v>
-      </c>
-      <c r="G360" s="2" t="inlineStr"/>
+        <v>46.76</v>
+      </c>
+      <c r="G360" s="3" t="n">
+        <v>22.5</v>
+      </c>
       <c r="H360" s="3" t="n">
         <v>2.15</v>
       </c>
       <c r="I360" s="4" t="n">
-        <v>-0.2756</v>
+        <v>0.1128</v>
       </c>
       <c r="J360" s="4" t="n">
-        <v>0.5871999999999999</v>
+        <v>-0.9066</v>
       </c>
       <c r="K360" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L360" s="2" t="inlineStr">
         <is>
-          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST KOBİ SANAYİ, BIST KONYA</t>
+          <t>BIST ULASTIRMA, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST ANA, BIST BALIKESİR</t>
         </is>
       </c>
       <c r="M360" s="2" t="inlineStr"/>
@@ -16153,44 +16155,42 @@
     <row r="361">
       <c r="A361" s="6" t="inlineStr">
         <is>
-          <t>MPARK</t>
+          <t>ERSU</t>
         </is>
       </c>
       <c r="B361" s="7" t="n">
-        <v>453</v>
+        <v>25.5</v>
       </c>
       <c r="C361" s="8" t="n">
-        <v>-0.0131</v>
+        <v>-0.0016</v>
       </c>
       <c r="D361" s="9" t="n">
-        <v>649990</v>
+        <v>542670</v>
       </c>
       <c r="E361" s="8" t="n">
-        <v>0.4234000000000001</v>
+        <v>0.7902</v>
       </c>
       <c r="F361" s="7" t="n">
-        <v>47.08</v>
-      </c>
-      <c r="G361" s="7" t="n">
-        <v>14.94</v>
-      </c>
+        <v>47.64</v>
+      </c>
+      <c r="G361" s="6" t="inlineStr"/>
       <c r="H361" s="7" t="n">
-        <v>2.16</v>
+        <v>2.15</v>
       </c>
       <c r="I361" s="8" t="n">
-        <v>0.1752</v>
+        <v>-0.2756</v>
       </c>
       <c r="J361" s="8" t="n">
-        <v>0.1408</v>
+        <v>0.5871999999999999</v>
       </c>
       <c r="K361" s="6" t="inlineStr">
         <is>
-          <t>Sağlık hizmetleri</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L361" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST SÜRDÜRÜLEBİLİRLİK, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK, STOXX Emerging Markets 1500</t>
+          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST KOBİ SANAYİ, BIST KONYA</t>
         </is>
       </c>
       <c r="M361" s="6" t="inlineStr"/>
@@ -16198,44 +16198,44 @@
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>MAALT</t>
-        </is>
-      </c>
-      <c r="B362" s="5" t="n">
-        <v>1350</v>
+          <t>MPARK</t>
+        </is>
+      </c>
+      <c r="B362" s="3" t="n">
+        <v>453</v>
       </c>
       <c r="C362" s="4" t="n">
-        <v>0.0143</v>
+        <v>-0.0131</v>
       </c>
       <c r="D362" s="5" t="n">
-        <v>156340</v>
+        <v>649990</v>
       </c>
       <c r="E362" s="4" t="n">
-        <v>0.4084</v>
+        <v>0.4234000000000001</v>
       </c>
       <c r="F362" s="3" t="n">
-        <v>65.42</v>
+        <v>47.08</v>
       </c>
       <c r="G362" s="3" t="n">
-        <v>354.02</v>
+        <v>14.94</v>
       </c>
       <c r="H362" s="3" t="n">
-        <v>2.17</v>
+        <v>2.16</v>
       </c>
       <c r="I362" s="4" t="n">
-        <v>0.0053</v>
+        <v>0.1752</v>
       </c>
       <c r="J362" s="4" t="n">
-        <v>-2.764</v>
+        <v>0.1408</v>
       </c>
       <c r="K362" s="2" t="inlineStr">
         <is>
-          <t>Tüketici hizmetleri</t>
+          <t>Sağlık hizmetleri</t>
         </is>
       </c>
       <c r="L362" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TURİZM, BIST HİZMETLER, BIST ANA, BIST ANTALYA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST SÜRDÜRÜLEBİLİRLİK, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK, STOXX Emerging Markets 1500</t>
         </is>
       </c>
       <c r="M362" s="2" t="inlineStr"/>
@@ -16243,44 +16243,44 @@
     <row r="363">
       <c r="A363" s="6" t="inlineStr">
         <is>
-          <t>EGPRO</t>
-        </is>
-      </c>
-      <c r="B363" s="7" t="n">
-        <v>40.32</v>
+          <t>MAALT</t>
+        </is>
+      </c>
+      <c r="B363" s="9" t="n">
+        <v>1350</v>
       </c>
       <c r="C363" s="8" t="n">
-        <v>-0.0098</v>
+        <v>0.0143</v>
       </c>
       <c r="D363" s="9" t="n">
-        <v>2370000</v>
+        <v>156340</v>
       </c>
       <c r="E363" s="8" t="n">
-        <v>0.1314</v>
+        <v>0.4084</v>
       </c>
       <c r="F363" s="7" t="n">
-        <v>54.04</v>
+        <v>65.42</v>
       </c>
       <c r="G363" s="7" t="n">
-        <v>18.02</v>
+        <v>354.02</v>
       </c>
       <c r="H363" s="7" t="n">
-        <v>2.18</v>
+        <v>2.17</v>
       </c>
       <c r="I363" s="8" t="n">
-        <v>0.1433</v>
+        <v>0.0053</v>
       </c>
       <c r="J363" s="8" t="n">
-        <v>-0.2049</v>
+        <v>-2.764</v>
       </c>
       <c r="K363" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Tüketici hizmetleri</t>
         </is>
       </c>
       <c r="L363" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST KATILIM TEMETTU, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TURİZM, BIST HİZMETLER, BIST ANA, BIST ANTALYA</t>
         </is>
       </c>
       <c r="M363" s="6" t="inlineStr"/>
@@ -16288,33 +16288,35 @@
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>RUZYE</t>
+          <t>EGPRO</t>
         </is>
       </c>
       <c r="B364" s="3" t="n">
-        <v>11.95</v>
+        <v>40.32</v>
       </c>
       <c r="C364" s="4" t="n">
-        <v>-0.0124</v>
+        <v>-0.0098</v>
       </c>
       <c r="D364" s="5" t="n">
-        <v>6110000</v>
+        <v>2370000</v>
       </c>
       <c r="E364" s="4" t="n">
-        <v>0.6456000000000001</v>
+        <v>0.1314</v>
       </c>
       <c r="F364" s="3" t="n">
-        <v>43.42</v>
-      </c>
-      <c r="G364" s="2" t="inlineStr"/>
+        <v>54.04</v>
+      </c>
+      <c r="G364" s="3" t="n">
+        <v>18.02</v>
+      </c>
       <c r="H364" s="3" t="n">
-        <v>2.19</v>
+        <v>2.18</v>
       </c>
       <c r="I364" s="4" t="n">
-        <v>-0.0029</v>
+        <v>0.1433</v>
       </c>
       <c r="J364" s="4" t="n">
-        <v>-3.8066</v>
+        <v>-0.2049</v>
       </c>
       <c r="K364" s="2" t="inlineStr">
         <is>
@@ -16323,7 +16325,7 @@
       </c>
       <c r="L364" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST MADENCİLİK, BIST ANA, BIST KOBİ SANAYİ, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST KATILIM TEMETTU, BIST İZMİR</t>
         </is>
       </c>
       <c r="M364" s="2" t="inlineStr"/>
@@ -16331,33 +16333,33 @@
     <row r="365">
       <c r="A365" s="6" t="inlineStr">
         <is>
-          <t>SONME</t>
+          <t>RUZYE</t>
         </is>
       </c>
       <c r="B365" s="7" t="n">
-        <v>139</v>
+        <v>11.95</v>
       </c>
       <c r="C365" s="8" t="n">
-        <v>0.0412</v>
+        <v>-0.0124</v>
       </c>
       <c r="D365" s="9" t="n">
-        <v>37780</v>
+        <v>6110000</v>
       </c>
       <c r="E365" s="8" t="n">
-        <v>0.0789</v>
+        <v>0.6456000000000001</v>
       </c>
       <c r="F365" s="7" t="n">
-        <v>52.58</v>
+        <v>43.42</v>
       </c>
       <c r="G365" s="6" t="inlineStr"/>
       <c r="H365" s="7" t="n">
-        <v>2.2</v>
+        <v>2.19</v>
       </c>
       <c r="I365" s="8" t="n">
-        <v>-0.08929999999999999</v>
+        <v>-0.0029</v>
       </c>
       <c r="J365" s="8" t="n">
-        <v>0.4032</v>
+        <v>-3.8066</v>
       </c>
       <c r="K365" s="6" t="inlineStr">
         <is>
@@ -16366,7 +16368,7 @@
       </c>
       <c r="L365" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST BURSA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST MADENCİLİK, BIST ANA, BIST KOBİ SANAYİ, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M365" s="6" t="inlineStr"/>
@@ -16374,126 +16376,124 @@
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>EKIZ</t>
+          <t>SONME</t>
         </is>
       </c>
       <c r="B366" s="3" t="n">
-        <v>85.2</v>
+        <v>139</v>
       </c>
       <c r="C366" s="4" t="n">
-        <v>-0.0139</v>
+        <v>0.0412</v>
       </c>
       <c r="D366" s="5" t="n">
-        <v>16390</v>
-      </c>
-      <c r="E366" s="2" t="inlineStr"/>
+        <v>37780</v>
+      </c>
+      <c r="E366" s="4" t="n">
+        <v>0.0789</v>
+      </c>
       <c r="F366" s="3" t="n">
-        <v>37.63</v>
+        <v>52.58</v>
       </c>
       <c r="G366" s="2" t="inlineStr"/>
       <c r="H366" s="3" t="n">
         <v>2.2</v>
       </c>
       <c r="I366" s="4" t="n">
-        <v>-0.1797</v>
+        <v>-0.08929999999999999</v>
       </c>
       <c r="J366" s="4" t="n">
-        <v>0.9384</v>
+        <v>0.4032</v>
       </c>
       <c r="K366" s="2" t="inlineStr">
         <is>
           <t>İşlenebilen endüstriler</t>
         </is>
       </c>
-      <c r="L366" s="2" t="inlineStr"/>
+      <c r="L366" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST BURSA</t>
+        </is>
+      </c>
       <c r="M366" s="2" t="inlineStr"/>
     </row>
     <row r="367">
       <c r="A367" s="6" t="inlineStr">
         <is>
-          <t>KLKIM</t>
+          <t>EKIZ</t>
         </is>
       </c>
       <c r="B367" s="7" t="n">
-        <v>31.34</v>
+        <v>85.2</v>
       </c>
       <c r="C367" s="8" t="n">
-        <v>-0.006999999999999999</v>
+        <v>-0.0139</v>
       </c>
       <c r="D367" s="9" t="n">
-        <v>2210000</v>
-      </c>
-      <c r="E367" s="8" t="n">
-        <v>0.2637</v>
-      </c>
+        <v>16390</v>
+      </c>
+      <c r="E367" s="6" t="inlineStr"/>
       <c r="F367" s="7" t="n">
-        <v>38.3</v>
-      </c>
-      <c r="G367" s="7" t="n">
-        <v>13.19</v>
-      </c>
+        <v>37.63</v>
+      </c>
+      <c r="G367" s="6" t="inlineStr"/>
       <c r="H367" s="7" t="n">
-        <v>2.22</v>
+        <v>2.2</v>
       </c>
       <c r="I367" s="8" t="n">
-        <v>0.2016</v>
+        <v>-0.1797</v>
       </c>
       <c r="J367" s="8" t="n">
-        <v>0.5552</v>
+        <v>0.9384</v>
       </c>
       <c r="K367" s="6" t="inlineStr">
         <is>
           <t>İşlenebilen endüstriler</t>
         </is>
       </c>
-      <c r="L367" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST İSTANBUL, BIST YILDIZ, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+      <c r="L367" s="6" t="inlineStr"/>
       <c r="M367" s="6" t="inlineStr"/>
     </row>
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>PCILT</t>
+          <t>KLKIM</t>
         </is>
       </c>
       <c r="B368" s="3" t="n">
-        <v>36.76</v>
+        <v>31.34</v>
       </c>
       <c r="C368" s="4" t="n">
-        <v>0.04019999999999999</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="D368" s="5" t="n">
-        <v>3390000</v>
+        <v>2210000</v>
       </c>
       <c r="E368" s="4" t="n">
-        <v>0.5865</v>
+        <v>0.2637</v>
       </c>
       <c r="F368" s="3" t="n">
-        <v>68.36</v>
+        <v>38.3</v>
       </c>
       <c r="G368" s="3" t="n">
-        <v>9.33</v>
+        <v>13.19</v>
       </c>
       <c r="H368" s="3" t="n">
         <v>2.22</v>
       </c>
       <c r="I368" s="4" t="n">
-        <v>0.2928</v>
+        <v>0.2016</v>
       </c>
       <c r="J368" s="4" t="n">
-        <v>0.6712</v>
+        <v>0.5552</v>
       </c>
       <c r="K368" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L368" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST İSTANBUL, BIST YILDIZ, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M368" s="2" t="inlineStr"/>
@@ -16501,42 +16501,44 @@
     <row r="369">
       <c r="A369" s="6" t="inlineStr">
         <is>
-          <t>SARKY</t>
+          <t>PCILT</t>
         </is>
       </c>
       <c r="B369" s="7" t="n">
-        <v>28.72</v>
+        <v>36.76</v>
       </c>
       <c r="C369" s="8" t="n">
-        <v>-0.0446</v>
+        <v>0.04019999999999999</v>
       </c>
       <c r="D369" s="9" t="n">
-        <v>22740000</v>
+        <v>3390000</v>
       </c>
       <c r="E369" s="8" t="n">
-        <v>0.6767</v>
+        <v>0.5865</v>
       </c>
       <c r="F369" s="7" t="n">
-        <v>49.95</v>
+        <v>68.36</v>
       </c>
       <c r="G369" s="7" t="n">
-        <v>80.63</v>
+        <v>9.33</v>
       </c>
       <c r="H369" s="7" t="n">
         <v>2.22</v>
       </c>
       <c r="I369" s="8" t="n">
-        <v>0.0343</v>
-      </c>
-      <c r="J369" s="6" t="inlineStr"/>
+        <v>0.2928</v>
+      </c>
+      <c r="J369" s="8" t="n">
+        <v>0.6712</v>
+      </c>
       <c r="K369" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L369" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU, BIST KATILIM 50, BIST KATILIM TEMETTU, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M369" s="6" t="inlineStr"/>
@@ -16544,34 +16546,34 @@
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>KLSER</t>
+          <t>SARKY</t>
         </is>
       </c>
       <c r="B370" s="3" t="n">
-        <v>27.94</v>
+        <v>28.72</v>
       </c>
       <c r="C370" s="4" t="n">
-        <v>-0.0092</v>
+        <v>-0.0446</v>
       </c>
       <c r="D370" s="5" t="n">
-        <v>2600000</v>
+        <v>22740000</v>
       </c>
       <c r="E370" s="4" t="n">
-        <v>0.2156</v>
+        <v>0.6767</v>
       </c>
       <c r="F370" s="3" t="n">
-        <v>51.72</v>
-      </c>
-      <c r="G370" s="2" t="inlineStr"/>
+        <v>49.95</v>
+      </c>
+      <c r="G370" s="3" t="n">
+        <v>80.63</v>
+      </c>
       <c r="H370" s="3" t="n">
-        <v>2.23</v>
+        <v>2.22</v>
       </c>
       <c r="I370" s="4" t="n">
-        <v>-0.4134</v>
-      </c>
-      <c r="J370" s="4" t="n">
-        <v>0.9543</v>
-      </c>
+        <v>0.0343</v>
+      </c>
+      <c r="J370" s="2" t="inlineStr"/>
       <c r="K370" s="2" t="inlineStr">
         <is>
           <t>Üretici imalatı</t>
@@ -16579,7 +16581,7 @@
       </c>
       <c r="L370" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST KATILIM TÜM, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU, BIST KATILIM 50, BIST KATILIM TEMETTU, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M370" s="2" t="inlineStr"/>
@@ -16587,44 +16589,42 @@
     <row r="371">
       <c r="A371" s="6" t="inlineStr">
         <is>
-          <t>MOPAS</t>
+          <t>KLSER</t>
         </is>
       </c>
       <c r="B371" s="7" t="n">
-        <v>39.76</v>
+        <v>27.94</v>
       </c>
       <c r="C371" s="8" t="n">
-        <v>-0.0035</v>
+        <v>-0.0092</v>
       </c>
       <c r="D371" s="9" t="n">
-        <v>5280000</v>
+        <v>2600000</v>
       </c>
       <c r="E371" s="8" t="n">
-        <v>0.21</v>
+        <v>0.2156</v>
       </c>
       <c r="F371" s="7" t="n">
-        <v>46.92</v>
-      </c>
-      <c r="G371" s="7" t="n">
-        <v>45.92</v>
-      </c>
+        <v>51.72</v>
+      </c>
+      <c r="G371" s="6" t="inlineStr"/>
       <c r="H371" s="7" t="n">
-        <v>2.24</v>
+        <v>2.23</v>
       </c>
       <c r="I371" s="8" t="n">
-        <v>0.0633</v>
+        <v>-0.4134</v>
       </c>
       <c r="J371" s="8" t="n">
-        <v>-0.2432</v>
+        <v>0.9543</v>
       </c>
       <c r="K371" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L371" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST TİCARET, BIST HİZMETLER, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST KATILIM TÜM, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK</t>
         </is>
       </c>
       <c r="M371" s="6" t="inlineStr"/>
@@ -16632,44 +16632,44 @@
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t>GARFA</t>
+          <t>MOPAS</t>
         </is>
       </c>
       <c r="B372" s="3" t="n">
-        <v>29.9</v>
+        <v>39.76</v>
       </c>
       <c r="C372" s="4" t="n">
-        <v>-0.0216</v>
+        <v>-0.0035</v>
       </c>
       <c r="D372" s="5" t="n">
-        <v>2960000</v>
+        <v>5280000</v>
       </c>
       <c r="E372" s="4" t="n">
-        <v>0.08380000000000001</v>
+        <v>0.21</v>
       </c>
       <c r="F372" s="3" t="n">
-        <v>50.06</v>
+        <v>46.92</v>
       </c>
       <c r="G372" s="3" t="n">
-        <v>5.58</v>
+        <v>45.92</v>
       </c>
       <c r="H372" s="3" t="n">
         <v>2.24</v>
       </c>
       <c r="I372" s="4" t="n">
-        <v>0.5025999999999999</v>
+        <v>0.0633</v>
       </c>
       <c r="J372" s="4" t="n">
-        <v>-0.121</v>
+        <v>-0.2432</v>
       </c>
       <c r="K372" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L372" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST FIN KIR FAKTÖRIZASYONU, BIST MALİ, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST TİCARET, BIST HİZMETLER, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M372" s="2" t="inlineStr"/>
@@ -19654,44 +19654,42 @@
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
         <is>
-          <t>SAYAS</t>
+          <t>ALKA</t>
         </is>
       </c>
       <c r="B442" s="3" t="n">
-        <v>55.8</v>
+        <v>10.46</v>
       </c>
       <c r="C442" s="4" t="n">
-        <v>0.0027</v>
+        <v>0.0029</v>
       </c>
       <c r="D442" s="5" t="n">
-        <v>2560000</v>
+        <v>6880000</v>
       </c>
       <c r="E442" s="4" t="n">
-        <v>0.5476</v>
+        <v>0.1937</v>
       </c>
       <c r="F442" s="3" t="n">
-        <v>59.89</v>
-      </c>
-      <c r="G442" s="3" t="n">
-        <v>28.44</v>
-      </c>
+        <v>42.24</v>
+      </c>
+      <c r="G442" s="2" t="inlineStr"/>
       <c r="H442" s="3" t="n">
-        <v>3.5</v>
+        <v>3.48</v>
       </c>
       <c r="I442" s="4" t="n">
-        <v>0.1475</v>
+        <v>-0.0728</v>
       </c>
       <c r="J442" s="4" t="n">
-        <v>-0.7215</v>
+        <v>0.2832</v>
       </c>
       <c r="K442" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L442" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST KATILIM TÜM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M442" s="2" t="inlineStr"/>
@@ -19699,44 +19697,44 @@
     <row r="443">
       <c r="A443" s="6" t="inlineStr">
         <is>
-          <t>LINK</t>
+          <t>SAYAS</t>
         </is>
       </c>
       <c r="B443" s="7" t="n">
-        <v>7.74</v>
+        <v>55.8</v>
       </c>
       <c r="C443" s="8" t="n">
-        <v>0.09939999999999999</v>
+        <v>0.0027</v>
       </c>
       <c r="D443" s="9" t="n">
-        <v>57130000</v>
+        <v>2560000</v>
       </c>
       <c r="E443" s="8" t="n">
-        <v>0.9937</v>
+        <v>0.5476</v>
       </c>
       <c r="F443" s="7" t="n">
-        <v>74.12</v>
+        <v>59.89</v>
       </c>
       <c r="G443" s="7" t="n">
-        <v>15.38</v>
+        <v>28.44</v>
       </c>
       <c r="H443" s="7" t="n">
-        <v>3.51</v>
+        <v>3.5</v>
       </c>
       <c r="I443" s="8" t="n">
-        <v>0.2897</v>
+        <v>0.1475</v>
       </c>
       <c r="J443" s="8" t="n">
-        <v>0.057</v>
+        <v>-0.7215</v>
       </c>
       <c r="K443" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L443" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST YILDIZ, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M443" s="6" t="inlineStr"/>
@@ -19744,44 +19742,44 @@
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
         <is>
-          <t>GENIL</t>
+          <t>LINK</t>
         </is>
       </c>
       <c r="B444" s="3" t="n">
-        <v>9.359999999999999</v>
+        <v>7.74</v>
       </c>
       <c r="C444" s="4" t="n">
-        <v>0.0152</v>
+        <v>0.09939999999999999</v>
       </c>
       <c r="D444" s="5" t="n">
-        <v>73480000</v>
+        <v>57130000</v>
       </c>
       <c r="E444" s="4" t="n">
-        <v>0.2412</v>
+        <v>0.9937</v>
       </c>
       <c r="F444" s="3" t="n">
-        <v>52.7</v>
+        <v>74.12</v>
       </c>
       <c r="G444" s="3" t="n">
-        <v>51.32</v>
+        <v>15.38</v>
       </c>
       <c r="H444" s="3" t="n">
-        <v>3.58</v>
+        <v>3.51</v>
       </c>
       <c r="I444" s="4" t="n">
-        <v>0.0815</v>
+        <v>0.2897</v>
       </c>
       <c r="J444" s="4" t="n">
-        <v>1.4915</v>
+        <v>0.057</v>
       </c>
       <c r="K444" s="2" t="inlineStr">
         <is>
-          <t>Sağlık teknolojisi</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L444" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU, BIST KATILIM 50, BIST KATILIM 30, BIST KATILIM TEMETTU, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST YILDIZ, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M444" s="2" t="inlineStr"/>
@@ -19789,42 +19787,44 @@
     <row r="445">
       <c r="A445" s="6" t="inlineStr">
         <is>
-          <t>BARMA</t>
+          <t>GENIL</t>
         </is>
       </c>
       <c r="B445" s="7" t="n">
-        <v>59.55</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="C445" s="8" t="n">
-        <v>-0.0092</v>
+        <v>0.0152</v>
       </c>
       <c r="D445" s="9" t="n">
-        <v>4450000</v>
+        <v>73480000</v>
       </c>
       <c r="E445" s="8" t="n">
-        <v>0.2</v>
+        <v>0.2412</v>
       </c>
       <c r="F445" s="7" t="n">
-        <v>55.16</v>
-      </c>
-      <c r="G445" s="6" t="inlineStr"/>
+        <v>52.7</v>
+      </c>
+      <c r="G445" s="7" t="n">
+        <v>51.32</v>
+      </c>
       <c r="H445" s="7" t="n">
-        <v>3.6</v>
+        <v>3.58</v>
       </c>
       <c r="I445" s="8" t="n">
-        <v>-0.005600000000000001</v>
+        <v>0.0815</v>
       </c>
       <c r="J445" s="8" t="n">
-        <v>-0.7101999999999999</v>
+        <v>1.4915</v>
       </c>
       <c r="K445" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Sağlık teknolojisi</t>
         </is>
       </c>
       <c r="L445" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST İZMİR</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU, BIST KATILIM 50, BIST KATILIM 30, BIST KATILIM TEMETTU, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M445" s="6" t="inlineStr"/>
@@ -19832,44 +19832,42 @@
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
         <is>
-          <t>LOGO</t>
+          <t>BARMA</t>
         </is>
       </c>
       <c r="B446" s="3" t="n">
-        <v>158.2</v>
+        <v>59.55</v>
       </c>
       <c r="C446" s="4" t="n">
-        <v>0.0347</v>
+        <v>-0.0092</v>
       </c>
       <c r="D446" s="5" t="n">
-        <v>928800</v>
+        <v>4450000</v>
       </c>
       <c r="E446" s="4" t="n">
-        <v>0.6459999999999999</v>
+        <v>0.2</v>
       </c>
       <c r="F446" s="3" t="n">
-        <v>57.46</v>
-      </c>
-      <c r="G446" s="3" t="n">
-        <v>19.26</v>
-      </c>
+        <v>55.16</v>
+      </c>
+      <c r="G446" s="2" t="inlineStr"/>
       <c r="H446" s="3" t="n">
-        <v>3.66</v>
+        <v>3.6</v>
       </c>
       <c r="I446" s="4" t="n">
-        <v>0.2184</v>
+        <v>-0.005600000000000001</v>
       </c>
       <c r="J446" s="4" t="n">
-        <v>-0.004500000000000001</v>
+        <v>-0.7101999999999999</v>
       </c>
       <c r="K446" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L446" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KATILIM TEMETTU, BIST KOCAELI, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST İZMİR</t>
         </is>
       </c>
       <c r="M446" s="2" t="inlineStr"/>
@@ -19877,42 +19875,44 @@
     <row r="447">
       <c r="A447" s="6" t="inlineStr">
         <is>
-          <t>ALKA</t>
+          <t>LOGO</t>
         </is>
       </c>
       <c r="B447" s="7" t="n">
-        <v>10.46</v>
+        <v>158.2</v>
       </c>
       <c r="C447" s="8" t="n">
-        <v>0.0029</v>
+        <v>0.0347</v>
       </c>
       <c r="D447" s="9" t="n">
-        <v>6880000</v>
+        <v>928800</v>
       </c>
       <c r="E447" s="8" t="n">
-        <v>0.1937</v>
+        <v>0.6459999999999999</v>
       </c>
       <c r="F447" s="7" t="n">
-        <v>42.24</v>
-      </c>
-      <c r="G447" s="6" t="inlineStr"/>
+        <v>57.46</v>
+      </c>
+      <c r="G447" s="7" t="n">
+        <v>19.26</v>
+      </c>
       <c r="H447" s="7" t="n">
-        <v>3.7</v>
+        <v>3.66</v>
       </c>
       <c r="I447" s="8" t="n">
-        <v>-0.0556</v>
+        <v>0.2184</v>
       </c>
       <c r="J447" s="8" t="n">
-        <v>-7.241000000000001</v>
+        <v>-0.004500000000000001</v>
       </c>
       <c r="K447" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L447" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST KATILIM TÜM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KATILIM TEMETTU, BIST KOCAELI, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK</t>
         </is>
       </c>
       <c r="M447" s="6" t="inlineStr"/>
@@ -25942,38 +25942,30 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>EKDMR</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>25.7</v>
+        <v>59.85</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.006999999999999999</v>
-      </c>
-      <c r="D588" s="5" t="n">
-        <v>527150</v>
-      </c>
-      <c r="E588" s="4" t="n">
-        <v>0.9698</v>
-      </c>
-      <c r="F588" s="3" t="n">
-        <v>45.64</v>
-      </c>
+        <v>0.0992</v>
+      </c>
+      <c r="D588" s="2" t="inlineStr"/>
+      <c r="E588" s="2" t="inlineStr"/>
+      <c r="F588" s="2" t="inlineStr"/>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
       <c r="I588" s="2" t="inlineStr"/>
-      <c r="J588" s="4" t="n">
-        <v>0.6453</v>
-      </c>
+      <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Enerji-dışı mineraller</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST HALKA ARZ, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25981,40 +25973,42 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>5.87</v>
+        <v>34.72</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>0.0731</v>
+        <v>-0.0012</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>18100000</v>
+        <v>4640000</v>
       </c>
       <c r="E589" s="8" t="n">
-        <v>0.1672</v>
+        <v>0.3528</v>
       </c>
       <c r="F589" s="7" t="n">
-        <v>49.01</v>
-      </c>
-      <c r="G589" s="6" t="inlineStr"/>
+        <v>46.16</v>
+      </c>
+      <c r="G589" s="7" t="n">
+        <v>13.72</v>
+      </c>
       <c r="H589" s="6" t="inlineStr"/>
       <c r="I589" s="8" t="n">
-        <v>-5.3262</v>
+        <v>0.1029</v>
       </c>
       <c r="J589" s="8" t="n">
-        <v>-4.2562</v>
+        <v>-1.4864</v>
       </c>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26022,21 +26016,21 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>191.9</v>
+        <v>2.6</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.0174</v>
+        <v>-0.0189</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>5800000</v>
+        <v>94430000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>55.81</v>
+        <v>42.83</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
@@ -26044,12 +26038,12 @@
       <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26057,23 +26051,21 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>36.38</v>
+        <v>17.67</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0022</v>
+        <v>-0.0172</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>23850000</v>
-      </c>
-      <c r="E591" s="8" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>21980000</v>
+      </c>
+      <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>68.22</v>
+        <v>36.71</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
@@ -26081,12 +26073,12 @@
       <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26129,71 +26121,81 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>12</v>
+        <v>5.87</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0.0345</v>
+        <v>0.0731</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>498860</v>
+        <v>18100000</v>
       </c>
       <c r="E593" s="8" t="n">
-        <v>0.95</v>
+        <v>0.1672</v>
       </c>
       <c r="F593" s="7" t="n">
-        <v>69.81999999999999</v>
+        <v>49.01</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
       <c r="I593" s="8" t="n">
-        <v>-23.6291</v>
+        <v>-5.3262</v>
       </c>
       <c r="J593" s="8" t="n">
-        <v>-0.4678</v>
+        <v>-4.2562</v>
       </c>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L593" s="6" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L593" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>2.6</v>
+        <v>129.6</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.0189</v>
+        <v>-0.0077</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>94430000</v>
-      </c>
-      <c r="E594" s="2" t="inlineStr"/>
+        <v>879570</v>
+      </c>
+      <c r="E594" s="4" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F594" s="3" t="n">
-        <v>42.83</v>
+        <v>41.79</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="2" t="inlineStr"/>
-      <c r="J594" s="2" t="inlineStr"/>
+      <c r="I594" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J594" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26201,40 +26203,40 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>129.6</v>
+        <v>2.4</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.0077</v>
+        <v>0</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>879570</v>
+        <v>16980000</v>
       </c>
       <c r="E595" s="8" t="n">
-        <v>0.1071</v>
+        <v>1</v>
       </c>
       <c r="F595" s="7" t="n">
-        <v>41.79</v>
+        <v>39.22</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
       <c r="I595" s="8" t="n">
-        <v>-3.6635</v>
+        <v>-191.6342</v>
       </c>
       <c r="J595" s="8" t="n">
-        <v>-0.4897</v>
+        <v>-0.8093</v>
       </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26242,56 +26244,56 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>13.92</v>
+        <v>70.25</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.0029</v>
+        <v>0.09939999999999999</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>19750000</v>
-      </c>
-      <c r="E596" s="2" t="inlineStr"/>
+        <v>42550</v>
+      </c>
+      <c r="E596" s="4" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F596" s="3" t="n">
-        <v>50.28</v>
+        <v>44.2</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
       <c r="I596" s="2" t="inlineStr"/>
-      <c r="J596" s="2" t="inlineStr"/>
+      <c r="J596" s="4" t="n">
+        <v>0.4928</v>
+      </c>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L596" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L596" s="2" t="inlineStr"/>
       <c r="M596" s="2" t="inlineStr"/>
     </row>
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>74.05</v>
+        <v>13.92</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>-0.0886</v>
+        <v>-0.0029</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>25520000</v>
+        <v>19750000</v>
       </c>
       <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>67.18000000000001</v>
+        <v>50.28</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
@@ -26299,12 +26301,12 @@
       <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26312,34 +26314,38 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>17.67</v>
+        <v>25.7</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0172</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>21980000</v>
-      </c>
-      <c r="E598" s="2" t="inlineStr"/>
+        <v>527150</v>
+      </c>
+      <c r="E598" s="4" t="n">
+        <v>0.9698</v>
+      </c>
       <c r="F598" s="3" t="n">
-        <v>36.71</v>
+        <v>45.64</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
       <c r="I598" s="2" t="inlineStr"/>
-      <c r="J598" s="2" t="inlineStr"/>
+      <c r="J598" s="4" t="n">
+        <v>0.6453</v>
+      </c>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26347,21 +26353,21 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>40.96</v>
+        <v>6.12</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.0039</v>
+        <v>0.009899999999999999</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>4380000</v>
+        <v>8660000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>50.43</v>
+        <v>54.27</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26369,34 +26375,30 @@
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L599" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L599" s="6" t="inlineStr"/>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>170.1</v>
+        <v>40.96</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>-0.023</v>
+        <v>0.0039</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>6070000</v>
+        <v>4380000</v>
       </c>
       <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>38.2</v>
+        <v>50.43</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
@@ -26404,12 +26406,12 @@
       <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26417,63 +26419,67 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>70.25</v>
+        <v>16.49</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.09939999999999999</v>
+        <v>0.005500000000000001</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>42550</v>
-      </c>
-      <c r="E601" s="8" t="n">
-        <v>0.58</v>
-      </c>
+        <v>28260000</v>
+      </c>
+      <c r="E601" s="6" t="inlineStr"/>
       <c r="F601" s="7" t="n">
-        <v>44.2</v>
+        <v>48.12</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
       <c r="I601" s="6" t="inlineStr"/>
-      <c r="J601" s="8" t="n">
-        <v>0.4928</v>
-      </c>
+      <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L601" s="6" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L601" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>245</v>
+        <v>12</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.0298</v>
+        <v>0.0345</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>9560</v>
+        <v>498860</v>
       </c>
       <c r="E602" s="4" t="n">
-        <v>0.2578</v>
+        <v>0.95</v>
       </c>
       <c r="F602" s="3" t="n">
-        <v>50.37</v>
+        <v>69.81999999999999</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
-      <c r="I602" s="2" t="inlineStr"/>
-      <c r="J602" s="2" t="inlineStr"/>
+      <c r="I602" s="4" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J602" s="4" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K602" s="2" t="inlineStr">
         <is>
           <t>İşlenebilen endüstriler</t>
@@ -26485,65 +26491,61 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>16.49</v>
+        <v>80.37</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.005500000000000001</v>
+        <v>-0.0042</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>28260000</v>
+        <v>11050000</v>
       </c>
       <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>48.12</v>
+        <v>49.24</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
       <c r="I603" s="6" t="inlineStr"/>
       <c r="J603" s="6" t="inlineStr"/>
-      <c r="K603" s="6" t="inlineStr">
-        <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L603" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+      <c r="K603" s="6" t="inlineStr"/>
+      <c r="L603" s="6" t="inlineStr"/>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>EKDMR</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>59.85</v>
+        <v>74.05</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0.0992</v>
-      </c>
-      <c r="D604" s="2" t="inlineStr"/>
+        <v>-0.0886</v>
+      </c>
+      <c r="D604" s="5" t="n">
+        <v>25520000</v>
+      </c>
       <c r="E604" s="2" t="inlineStr"/>
-      <c r="F604" s="2" t="inlineStr"/>
+      <c r="F604" s="3" t="n">
+        <v>67.18000000000001</v>
+      </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
       <c r="I604" s="2" t="inlineStr"/>
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST HALKA ARZ, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26551,21 +26553,21 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>6.12</v>
+        <v>39.6</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.009899999999999999</v>
+        <v>-0.0365</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>8660000</v>
+        <v>11700000</v>
       </c>
       <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>54.27</v>
+        <v>59.52</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
@@ -26573,30 +26575,36 @@
       <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L605" s="6" t="inlineStr"/>
+          <t>Üretici imalatı</t>
+        </is>
+      </c>
+      <c r="L605" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+        </is>
+      </c>
       <c r="M605" s="6" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>77</v>
+        <v>245</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.0158</v>
+        <v>0.0298</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>137290</v>
-      </c>
-      <c r="E606" s="2" t="inlineStr"/>
+        <v>9560</v>
+      </c>
+      <c r="E606" s="4" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F606" s="3" t="n">
-        <v>28.48</v>
+        <v>50.37</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
@@ -26604,7 +26612,7 @@
       <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr"/>
@@ -26613,21 +26621,21 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>39.6</v>
+        <v>77</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.0365</v>
+        <v>0.0158</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>11700000</v>
+        <v>137290</v>
       </c>
       <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>59.52</v>
+        <v>28.48</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26635,53 +26643,45 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L607" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L607" s="6" t="inlineStr"/>
       <c r="M607" s="6" t="inlineStr"/>
     </row>
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>2.4</v>
+        <v>36.38</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>0</v>
+        <v>0.0022</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>16980000</v>
+        <v>23850000</v>
       </c>
       <c r="E608" s="4" t="n">
-        <v>1</v>
+        <v>0.2667</v>
       </c>
       <c r="F608" s="3" t="n">
-        <v>39.22</v>
+        <v>68.22</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
-      <c r="I608" s="4" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J608" s="4" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I608" s="2" t="inlineStr"/>
+      <c r="J608" s="2" t="inlineStr"/>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L608" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M608" s="2" t="inlineStr"/>
@@ -26689,34 +26689,38 @@
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>32.18</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>0.0255</v>
+        <v>0.0121</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>17120000</v>
-      </c>
-      <c r="E609" s="6" t="inlineStr"/>
+        <v>562280</v>
+      </c>
+      <c r="E609" s="8" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F609" s="7" t="n">
-        <v>65.51000000000001</v>
+        <v>54.15</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
       <c r="I609" s="6" t="inlineStr"/>
-      <c r="J609" s="6" t="inlineStr"/>
+      <c r="J609" s="8" t="n">
+        <v>0.1431</v>
+      </c>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L609" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M609" s="6" t="inlineStr"/>
@@ -26724,65 +26728,69 @@
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>80.37</v>
+        <v>191.9</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>-0.0042</v>
+        <v>-0.0174</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>11050000</v>
+        <v>5800000</v>
       </c>
       <c r="E610" s="2" t="inlineStr"/>
       <c r="F610" s="3" t="n">
-        <v>49.24</v>
+        <v>55.81</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
       <c r="I610" s="2" t="inlineStr"/>
       <c r="J610" s="2" t="inlineStr"/>
-      <c r="K610" s="2" t="inlineStr"/>
-      <c r="L610" s="2" t="inlineStr"/>
+      <c r="K610" s="2" t="inlineStr">
+        <is>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L610" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+        </is>
+      </c>
       <c r="M610" s="2" t="inlineStr"/>
     </row>
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>67.15000000000001</v>
+        <v>170.1</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>0.0121</v>
+        <v>-0.023</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>562280</v>
-      </c>
-      <c r="E611" s="8" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>6070000</v>
+      </c>
+      <c r="E611" s="6" t="inlineStr"/>
       <c r="F611" s="7" t="n">
-        <v>54.15</v>
+        <v>38.2</v>
       </c>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
       <c r="I611" s="6" t="inlineStr"/>
-      <c r="J611" s="8" t="n">
-        <v>0.1431</v>
-      </c>
+      <c r="J611" s="6" t="inlineStr"/>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L611" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M611" s="6" t="inlineStr"/>
@@ -26790,42 +26798,34 @@
     <row r="612">
       <c r="A612" s="2" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B612" s="3" t="n">
-        <v>34.72</v>
+        <v>32.18</v>
       </c>
       <c r="C612" s="4" t="n">
-        <v>-0.0012</v>
+        <v>0.0255</v>
       </c>
       <c r="D612" s="5" t="n">
-        <v>4640000</v>
-      </c>
-      <c r="E612" s="4" t="n">
-        <v>0.3528</v>
-      </c>
+        <v>17120000</v>
+      </c>
+      <c r="E612" s="2" t="inlineStr"/>
       <c r="F612" s="3" t="n">
-        <v>46.16</v>
-      </c>
-      <c r="G612" s="3" t="n">
-        <v>13.72</v>
-      </c>
+        <v>65.51000000000001</v>
+      </c>
+      <c r="G612" s="2" t="inlineStr"/>
       <c r="H612" s="2" t="inlineStr"/>
-      <c r="I612" s="4" t="n">
-        <v>0.1029</v>
-      </c>
-      <c r="J612" s="4" t="n">
-        <v>-1.4864</v>
-      </c>
+      <c r="I612" s="2" t="inlineStr"/>
+      <c r="J612" s="2" t="inlineStr"/>
       <c r="K612" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L612" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M612" s="2" t="inlineStr"/>
@@ -26852,7 +26852,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>27.05.2026 12:30</t>
+          <t>27.05.2026 13:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 27.05.2026 14:30 | 611 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-27.xlsx
+++ b/data/bist_screener_2026-05-27.xlsx
@@ -25942,108 +25942,108 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>EKDMR</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>59.85</v>
+        <v>77</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.0992</v>
-      </c>
-      <c r="D588" s="2" t="inlineStr"/>
+        <v>0.0158</v>
+      </c>
+      <c r="D588" s="5" t="n">
+        <v>137290</v>
+      </c>
       <c r="E588" s="2" t="inlineStr"/>
-      <c r="F588" s="2" t="inlineStr"/>
+      <c r="F588" s="3" t="n">
+        <v>28.48</v>
+      </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
       <c r="I588" s="2" t="inlineStr"/>
       <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
-        </is>
-      </c>
-      <c r="L588" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST HALKA ARZ, BIST YILDIZ</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L588" s="2" t="inlineStr"/>
       <c r="M588" s="2" t="inlineStr"/>
     </row>
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>34.72</v>
+        <v>12</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0012</v>
+        <v>0.0345</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>4640000</v>
+        <v>498860</v>
       </c>
       <c r="E589" s="8" t="n">
-        <v>0.3528</v>
+        <v>0.95</v>
       </c>
       <c r="F589" s="7" t="n">
-        <v>46.16</v>
-      </c>
-      <c r="G589" s="7" t="n">
-        <v>13.72</v>
-      </c>
+        <v>69.81999999999999</v>
+      </c>
+      <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
       <c r="I589" s="8" t="n">
-        <v>0.1029</v>
+        <v>-23.6291</v>
       </c>
       <c r="J589" s="8" t="n">
-        <v>-1.4864</v>
+        <v>-0.4678</v>
       </c>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
-        </is>
-      </c>
-      <c r="L589" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L589" s="6" t="inlineStr"/>
       <c r="M589" s="6" t="inlineStr"/>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>2.6</v>
+        <v>129.6</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.0189</v>
+        <v>-0.0077</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>94430000</v>
-      </c>
-      <c r="E590" s="2" t="inlineStr"/>
+        <v>879570</v>
+      </c>
+      <c r="E590" s="4" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F590" s="3" t="n">
-        <v>42.83</v>
+        <v>41.79</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
-      <c r="I590" s="2" t="inlineStr"/>
-      <c r="J590" s="2" t="inlineStr"/>
+      <c r="I590" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J590" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26051,21 +26051,23 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>17.67</v>
+        <v>36.38</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>-0.0172</v>
+        <v>0.0022</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>21980000</v>
-      </c>
-      <c r="E591" s="6" t="inlineStr"/>
+        <v>23850000</v>
+      </c>
+      <c r="E591" s="8" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F591" s="7" t="n">
-        <v>36.71</v>
+        <v>68.22</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
@@ -26073,12 +26075,12 @@
       <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26086,21 +26088,21 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>16.3</v>
+        <v>191.9</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.0151</v>
+        <v>-0.0174</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>30420000</v>
+        <v>5800000</v>
       </c>
       <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>45.98</v>
+        <v>55.81</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
@@ -26113,7 +26115,7 @@
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26121,32 +26123,26 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>5.87</v>
+        <v>2.6</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0.0731</v>
+        <v>-0.0189</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>18100000</v>
-      </c>
-      <c r="E593" s="8" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>94430000</v>
+      </c>
+      <c r="E593" s="6" t="inlineStr"/>
       <c r="F593" s="7" t="n">
-        <v>49.01</v>
+        <v>42.83</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J593" s="8" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I593" s="6" t="inlineStr"/>
+      <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -26154,7 +26150,7 @@
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26162,40 +26158,30 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>EKDMR</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>129.6</v>
+        <v>59.85</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.0077</v>
-      </c>
-      <c r="D594" s="5" t="n">
-        <v>879570</v>
-      </c>
-      <c r="E594" s="4" t="n">
-        <v>0.1071</v>
-      </c>
-      <c r="F594" s="3" t="n">
-        <v>41.79</v>
-      </c>
+        <v>0.0992</v>
+      </c>
+      <c r="D594" s="2" t="inlineStr"/>
+      <c r="E594" s="2" t="inlineStr"/>
+      <c r="F594" s="2" t="inlineStr"/>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J594" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I594" s="2" t="inlineStr"/>
+      <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Enerji-dışı mineraller</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST HALKA ARZ, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26203,40 +26189,34 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>2.4</v>
+        <v>74.05</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0</v>
+        <v>-0.0886</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>16980000</v>
-      </c>
-      <c r="E595" s="8" t="n">
-        <v>1</v>
-      </c>
+        <v>25520000</v>
+      </c>
+      <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="7" t="n">
-        <v>39.22</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
-      <c r="I595" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J595" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I595" s="6" t="inlineStr"/>
+      <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26279,34 +26259,42 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>13.92</v>
+        <v>34.72</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>-0.0029</v>
+        <v>-0.0012</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>19750000</v>
-      </c>
-      <c r="E597" s="6" t="inlineStr"/>
+        <v>4640000</v>
+      </c>
+      <c r="E597" s="8" t="n">
+        <v>0.3528</v>
+      </c>
       <c r="F597" s="7" t="n">
-        <v>50.28</v>
-      </c>
-      <c r="G597" s="6" t="inlineStr"/>
+        <v>46.16</v>
+      </c>
+      <c r="G597" s="7" t="n">
+        <v>13.72</v>
+      </c>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="6" t="inlineStr"/>
-      <c r="J597" s="6" t="inlineStr"/>
+      <c r="I597" s="8" t="n">
+        <v>0.1029</v>
+      </c>
+      <c r="J597" s="8" t="n">
+        <v>-1.4864</v>
+      </c>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26314,38 +26302,38 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>25.7</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.006999999999999999</v>
+        <v>0.0121</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>527150</v>
+        <v>562280</v>
       </c>
       <c r="E598" s="4" t="n">
-        <v>0.9698</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F598" s="3" t="n">
-        <v>45.64</v>
+        <v>54.15</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
       <c r="I598" s="2" t="inlineStr"/>
       <c r="J598" s="4" t="n">
-        <v>0.6453</v>
+        <v>0.1431</v>
       </c>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26384,21 +26372,21 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>40.96</v>
+        <v>16.3</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.0039</v>
+        <v>-0.0151</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>4380000</v>
+        <v>30420000</v>
       </c>
       <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>50.43</v>
+        <v>45.98</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
@@ -26406,12 +26394,12 @@
       <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26419,26 +26407,32 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>16.49</v>
+        <v>5.87</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.005500000000000001</v>
+        <v>0.0731</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>28260000</v>
-      </c>
-      <c r="E601" s="6" t="inlineStr"/>
+        <v>18100000</v>
+      </c>
+      <c r="E601" s="8" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F601" s="7" t="n">
-        <v>48.12</v>
+        <v>49.01</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="6" t="inlineStr"/>
-      <c r="J601" s="6" t="inlineStr"/>
+      <c r="I601" s="8" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J601" s="8" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K601" s="6" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -26446,7 +26440,7 @@
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26454,85 +26448,91 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>12</v>
+        <v>16.49</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.0345</v>
+        <v>0.005500000000000001</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>498860</v>
-      </c>
-      <c r="E602" s="4" t="n">
-        <v>0.95</v>
-      </c>
+        <v>28260000</v>
+      </c>
+      <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>69.81999999999999</v>
+        <v>48.12</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
-      <c r="I602" s="4" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J602" s="4" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I602" s="2" t="inlineStr"/>
+      <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L602" s="2" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L602" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>80.37</v>
+        <v>32.18</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.0042</v>
+        <v>0.0255</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>11050000</v>
+        <v>17120000</v>
       </c>
       <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>49.24</v>
+        <v>65.51000000000001</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
       <c r="I603" s="6" t="inlineStr"/>
       <c r="J603" s="6" t="inlineStr"/>
-      <c r="K603" s="6" t="inlineStr"/>
-      <c r="L603" s="6" t="inlineStr"/>
+      <c r="K603" s="6" t="inlineStr">
+        <is>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
+        </is>
+      </c>
+      <c r="L603" s="6" t="inlineStr">
+        <is>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>74.05</v>
+        <v>170.1</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0886</v>
+        <v>-0.023</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>25520000</v>
+        <v>6070000</v>
       </c>
       <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>67.18000000000001</v>
+        <v>38.2</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26540,12 +26540,12 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26553,34 +26553,38 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>39.6</v>
+        <v>25.7</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.0365</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>11700000</v>
-      </c>
-      <c r="E605" s="6" t="inlineStr"/>
+        <v>527150</v>
+      </c>
+      <c r="E605" s="8" t="n">
+        <v>0.9698</v>
+      </c>
       <c r="F605" s="7" t="n">
-        <v>59.52</v>
+        <v>45.64</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
       <c r="I605" s="6" t="inlineStr"/>
-      <c r="J605" s="6" t="inlineStr"/>
+      <c r="J605" s="8" t="n">
+        <v>0.6453</v>
+      </c>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26588,23 +26592,21 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>245</v>
+        <v>40.96</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.0298</v>
+        <v>0.0039</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>9560</v>
-      </c>
-      <c r="E606" s="4" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>4380000</v>
+      </c>
+      <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>50.37</v>
+        <v>50.43</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
@@ -26612,30 +26614,34 @@
       <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L606" s="2" t="inlineStr"/>
+          <t>Dayanıklı tüketim malları</t>
+        </is>
+      </c>
+      <c r="L606" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+        </is>
+      </c>
       <c r="M606" s="2" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>77</v>
+        <v>13.92</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>0.0158</v>
+        <v>-0.0029</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>137290</v>
+        <v>19750000</v>
       </c>
       <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>28.48</v>
+        <v>50.28</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26643,32 +26649,36 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L607" s="6" t="inlineStr"/>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L607" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M607" s="6" t="inlineStr"/>
     </row>
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>36.38</v>
+        <v>245</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>0.0022</v>
+        <v>0.0298</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>23850000</v>
+        <v>9560</v>
       </c>
       <c r="E608" s="4" t="n">
-        <v>0.2667</v>
+        <v>0.2578</v>
       </c>
       <c r="F608" s="3" t="n">
-        <v>68.22</v>
+        <v>50.37</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
@@ -26676,51 +26686,43 @@
       <c r="J608" s="2" t="inlineStr"/>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L608" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L608" s="2" t="inlineStr"/>
       <c r="M608" s="2" t="inlineStr"/>
     </row>
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>67.15000000000001</v>
+        <v>39.6</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>0.0121</v>
+        <v>-0.0365</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>562280</v>
-      </c>
-      <c r="E609" s="8" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>11700000</v>
+      </c>
+      <c r="E609" s="6" t="inlineStr"/>
       <c r="F609" s="7" t="n">
-        <v>54.15</v>
+        <v>59.52</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
       <c r="I609" s="6" t="inlineStr"/>
-      <c r="J609" s="8" t="n">
-        <v>0.1431</v>
-      </c>
+      <c r="J609" s="6" t="inlineStr"/>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L609" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M609" s="6" t="inlineStr"/>
@@ -26728,69 +26730,67 @@
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>191.9</v>
+        <v>80.37</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>-0.0174</v>
+        <v>-0.0042</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>5800000</v>
+        <v>11050000</v>
       </c>
       <c r="E610" s="2" t="inlineStr"/>
       <c r="F610" s="3" t="n">
-        <v>55.81</v>
+        <v>49.24</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
       <c r="I610" s="2" t="inlineStr"/>
       <c r="J610" s="2" t="inlineStr"/>
-      <c r="K610" s="2" t="inlineStr">
-        <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L610" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
-        </is>
-      </c>
+      <c r="K610" s="2" t="inlineStr"/>
+      <c r="L610" s="2" t="inlineStr"/>
       <c r="M610" s="2" t="inlineStr"/>
     </row>
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>170.1</v>
+        <v>2.4</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>-0.023</v>
+        <v>0</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>6070000</v>
-      </c>
-      <c r="E611" s="6" t="inlineStr"/>
+        <v>16980000</v>
+      </c>
+      <c r="E611" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="F611" s="7" t="n">
-        <v>38.2</v>
+        <v>39.22</v>
       </c>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
-      <c r="I611" s="6" t="inlineStr"/>
-      <c r="J611" s="6" t="inlineStr"/>
+      <c r="I611" s="8" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J611" s="8" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L611" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M611" s="6" t="inlineStr"/>
@@ -26798,21 +26798,21 @@
     <row r="612">
       <c r="A612" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B612" s="3" t="n">
-        <v>32.18</v>
+        <v>17.67</v>
       </c>
       <c r="C612" s="4" t="n">
-        <v>0.0255</v>
+        <v>-0.0172</v>
       </c>
       <c r="D612" s="5" t="n">
-        <v>17120000</v>
+        <v>21980000</v>
       </c>
       <c r="E612" s="2" t="inlineStr"/>
       <c r="F612" s="3" t="n">
-        <v>65.51000000000001</v>
+        <v>36.71</v>
       </c>
       <c r="G612" s="2" t="inlineStr"/>
       <c r="H612" s="2" t="inlineStr"/>
@@ -26820,12 +26820,12 @@
       <c r="J612" s="2" t="inlineStr"/>
       <c r="K612" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L612" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M612" s="2" t="inlineStr"/>
@@ -26852,7 +26852,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>27.05.2026 13:30</t>
+          <t>27.05.2026 14:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 27.05.2026 15:30 | 611 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-27.xlsx
+++ b/data/bist_screener_2026-05-27.xlsx
@@ -25942,21 +25942,23 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>77</v>
+        <v>36.38</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.0158</v>
+        <v>0.0022</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>137290</v>
-      </c>
-      <c r="E588" s="2" t="inlineStr"/>
+        <v>23850000</v>
+      </c>
+      <c r="E588" s="4" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F588" s="3" t="n">
-        <v>28.48</v>
+        <v>68.22</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
@@ -25964,86 +25966,82 @@
       <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L588" s="2" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L588" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M588" s="2" t="inlineStr"/>
     </row>
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>12</v>
+        <v>17.67</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>0.0345</v>
+        <v>-0.0172</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>498860</v>
-      </c>
-      <c r="E589" s="8" t="n">
-        <v>0.95</v>
-      </c>
+        <v>21980000</v>
+      </c>
+      <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>69.81999999999999</v>
+        <v>36.71</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
-      <c r="I589" s="8" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J589" s="8" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I589" s="6" t="inlineStr"/>
+      <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L589" s="6" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L589" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M589" s="6" t="inlineStr"/>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>129.6</v>
+        <v>74.05</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.0077</v>
+        <v>-0.0886</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>879570</v>
-      </c>
-      <c r="E590" s="4" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>25520000</v>
+      </c>
+      <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>41.79</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
-      <c r="I590" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J590" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I590" s="2" t="inlineStr"/>
+      <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26051,23 +26049,21 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>36.38</v>
+        <v>40.96</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0022</v>
+        <v>0.0039</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>23850000</v>
-      </c>
-      <c r="E591" s="8" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>4380000</v>
+      </c>
+      <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>68.22</v>
+        <v>50.43</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
@@ -26075,12 +26071,12 @@
       <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26088,36 +26084,38 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>191.9</v>
+        <v>12</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.0174</v>
+        <v>0.0345</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>5800000</v>
-      </c>
-      <c r="E592" s="2" t="inlineStr"/>
+        <v>498860</v>
+      </c>
+      <c r="E592" s="4" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F592" s="3" t="n">
-        <v>55.81</v>
+        <v>69.81999999999999</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
-      <c r="I592" s="2" t="inlineStr"/>
-      <c r="J592" s="2" t="inlineStr"/>
+      <c r="I592" s="4" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J592" s="4" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L592" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr"/>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
@@ -26158,30 +26156,42 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>EKDMR</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>59.85</v>
+        <v>34.72</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0.0992</v>
-      </c>
-      <c r="D594" s="2" t="inlineStr"/>
-      <c r="E594" s="2" t="inlineStr"/>
-      <c r="F594" s="2" t="inlineStr"/>
-      <c r="G594" s="2" t="inlineStr"/>
+        <v>-0.0012</v>
+      </c>
+      <c r="D594" s="5" t="n">
+        <v>4640000</v>
+      </c>
+      <c r="E594" s="4" t="n">
+        <v>0.3528</v>
+      </c>
+      <c r="F594" s="3" t="n">
+        <v>46.16</v>
+      </c>
+      <c r="G594" s="3" t="n">
+        <v>13.72</v>
+      </c>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="2" t="inlineStr"/>
-      <c r="J594" s="2" t="inlineStr"/>
+      <c r="I594" s="4" t="n">
+        <v>0.1029</v>
+      </c>
+      <c r="J594" s="4" t="n">
+        <v>-1.4864</v>
+      </c>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST HALKA ARZ, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26189,34 +26199,40 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>74.05</v>
+        <v>5.87</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.0886</v>
+        <v>0.0731</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>25520000</v>
-      </c>
-      <c r="E595" s="6" t="inlineStr"/>
+        <v>18100000</v>
+      </c>
+      <c r="E595" s="8" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F595" s="7" t="n">
-        <v>67.18000000000001</v>
+        <v>49.01</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
-      <c r="I595" s="6" t="inlineStr"/>
-      <c r="J595" s="6" t="inlineStr"/>
+      <c r="I595" s="8" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J595" s="8" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26224,33 +26240,29 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>70.25</v>
+        <v>77</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.09939999999999999</v>
+        <v>0.0158</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>42550</v>
-      </c>
-      <c r="E596" s="4" t="n">
-        <v>0.58</v>
-      </c>
+        <v>137290</v>
+      </c>
+      <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>44.2</v>
+        <v>28.48</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
       <c r="I596" s="2" t="inlineStr"/>
-      <c r="J596" s="4" t="n">
-        <v>0.4928</v>
-      </c>
+      <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr"/>
@@ -26259,42 +26271,38 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>34.72</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>-0.0012</v>
+        <v>0.0121</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>4640000</v>
+        <v>562280</v>
       </c>
       <c r="E597" s="8" t="n">
-        <v>0.3528</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F597" s="7" t="n">
-        <v>46.16</v>
-      </c>
-      <c r="G597" s="7" t="n">
-        <v>13.72</v>
-      </c>
+        <v>54.15</v>
+      </c>
+      <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="8" t="n">
-        <v>0.1029</v>
-      </c>
+      <c r="I597" s="6" t="inlineStr"/>
       <c r="J597" s="8" t="n">
-        <v>-1.4864</v>
+        <v>0.1431</v>
       </c>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26302,38 +26310,34 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>67.15000000000001</v>
+        <v>39.6</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>0.0121</v>
+        <v>-0.0365</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>562280</v>
-      </c>
-      <c r="E598" s="4" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>11700000</v>
+      </c>
+      <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>54.15</v>
+        <v>59.52</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
       <c r="I598" s="2" t="inlineStr"/>
-      <c r="J598" s="4" t="n">
-        <v>0.1431</v>
-      </c>
+      <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26372,21 +26376,21 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>16.3</v>
+        <v>191.9</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>-0.0151</v>
+        <v>-0.0174</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>30420000</v>
+        <v>5800000</v>
       </c>
       <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>45.98</v>
+        <v>55.81</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
@@ -26399,7 +26403,7 @@
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26407,75 +26411,63 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>5.87</v>
+        <v>245</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.0731</v>
+        <v>0.0298</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>18100000</v>
+        <v>9560</v>
       </c>
       <c r="E601" s="8" t="n">
-        <v>0.1672</v>
+        <v>0.2578</v>
       </c>
       <c r="F601" s="7" t="n">
-        <v>49.01</v>
+        <v>50.37</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J601" s="8" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I601" s="6" t="inlineStr"/>
+      <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L601" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L601" s="6" t="inlineStr"/>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>EKDMR</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>16.49</v>
+        <v>59.85</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.005500000000000001</v>
-      </c>
-      <c r="D602" s="5" t="n">
-        <v>28260000</v>
-      </c>
+        <v>0.0992</v>
+      </c>
+      <c r="D602" s="2" t="inlineStr"/>
       <c r="E602" s="2" t="inlineStr"/>
-      <c r="F602" s="3" t="n">
-        <v>48.12</v>
-      </c>
+      <c r="F602" s="2" t="inlineStr"/>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
       <c r="I602" s="2" t="inlineStr"/>
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Enerji-dışı mineraller</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST HALKA ARZ, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26483,34 +26475,40 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>32.18</v>
+        <v>129.6</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0255</v>
+        <v>-0.0077</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>17120000</v>
-      </c>
-      <c r="E603" s="6" t="inlineStr"/>
+        <v>879570</v>
+      </c>
+      <c r="E603" s="8" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F603" s="7" t="n">
-        <v>65.51000000000001</v>
+        <v>41.79</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="6" t="inlineStr"/>
-      <c r="J603" s="6" t="inlineStr"/>
+      <c r="I603" s="8" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J603" s="8" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26518,21 +26516,21 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>170.1</v>
+        <v>32.18</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.023</v>
+        <v>0.0255</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>6070000</v>
+        <v>17120000</v>
       </c>
       <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>38.2</v>
+        <v>65.51000000000001</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26540,12 +26538,12 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26553,38 +26551,40 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>25.7</v>
+        <v>2.4</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.006999999999999999</v>
+        <v>0</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>527150</v>
+        <v>16980000</v>
       </c>
       <c r="E605" s="8" t="n">
-        <v>0.9698</v>
+        <v>1</v>
       </c>
       <c r="F605" s="7" t="n">
-        <v>45.64</v>
+        <v>39.22</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
-      <c r="I605" s="6" t="inlineStr"/>
+      <c r="I605" s="8" t="n">
+        <v>-191.6342</v>
+      </c>
       <c r="J605" s="8" t="n">
-        <v>0.6453</v>
+        <v>-0.8093</v>
       </c>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26592,21 +26592,21 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>40.96</v>
+        <v>13.92</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.0039</v>
+        <v>-0.0029</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>4380000</v>
+        <v>19750000</v>
       </c>
       <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>50.43</v>
+        <v>50.28</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
@@ -26614,12 +26614,12 @@
       <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26627,21 +26627,21 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>13.92</v>
+        <v>170.1</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.0029</v>
+        <v>-0.023</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>19750000</v>
+        <v>6070000</v>
       </c>
       <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>50.28</v>
+        <v>38.2</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26649,12 +26649,12 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26662,31 +26662,33 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>245</v>
+        <v>70.25</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>0.0298</v>
+        <v>0.09939999999999999</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>9560</v>
+        <v>42550</v>
       </c>
       <c r="E608" s="4" t="n">
-        <v>0.2578</v>
+        <v>0.58</v>
       </c>
       <c r="F608" s="3" t="n">
-        <v>50.37</v>
+        <v>44.2</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
       <c r="I608" s="2" t="inlineStr"/>
-      <c r="J608" s="2" t="inlineStr"/>
+      <c r="J608" s="4" t="n">
+        <v>0.4928</v>
+      </c>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Taşımacılık</t>
         </is>
       </c>
       <c r="L608" s="2" t="inlineStr"/>
@@ -26695,102 +26697,96 @@
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>39.6</v>
+        <v>80.37</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>-0.0365</v>
+        <v>-0.0042</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>11700000</v>
+        <v>11050000</v>
       </c>
       <c r="E609" s="6" t="inlineStr"/>
       <c r="F609" s="7" t="n">
-        <v>59.52</v>
+        <v>49.24</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
       <c r="I609" s="6" t="inlineStr"/>
       <c r="J609" s="6" t="inlineStr"/>
-      <c r="K609" s="6" t="inlineStr">
-        <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L609" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+      <c r="K609" s="6" t="inlineStr"/>
+      <c r="L609" s="6" t="inlineStr"/>
       <c r="M609" s="6" t="inlineStr"/>
     </row>
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>80.37</v>
+        <v>16.3</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>-0.0042</v>
+        <v>-0.0151</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>11050000</v>
+        <v>30420000</v>
       </c>
       <c r="E610" s="2" t="inlineStr"/>
       <c r="F610" s="3" t="n">
-        <v>49.24</v>
+        <v>45.98</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
       <c r="I610" s="2" t="inlineStr"/>
       <c r="J610" s="2" t="inlineStr"/>
-      <c r="K610" s="2" t="inlineStr"/>
-      <c r="L610" s="2" t="inlineStr"/>
+      <c r="K610" s="2" t="inlineStr">
+        <is>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L610" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+        </is>
+      </c>
       <c r="M610" s="2" t="inlineStr"/>
     </row>
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>2.4</v>
+        <v>16.49</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>0</v>
+        <v>0.005500000000000001</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>16980000</v>
-      </c>
-      <c r="E611" s="8" t="n">
-        <v>1</v>
-      </c>
+        <v>28260000</v>
+      </c>
+      <c r="E611" s="6" t="inlineStr"/>
       <c r="F611" s="7" t="n">
-        <v>39.22</v>
+        <v>48.12</v>
       </c>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
-      <c r="I611" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J611" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I611" s="6" t="inlineStr"/>
+      <c r="J611" s="6" t="inlineStr"/>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L611" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M611" s="6" t="inlineStr"/>
@@ -26798,34 +26794,38 @@
     <row r="612">
       <c r="A612" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B612" s="3" t="n">
-        <v>17.67</v>
+        <v>25.7</v>
       </c>
       <c r="C612" s="4" t="n">
-        <v>-0.0172</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="D612" s="5" t="n">
-        <v>21980000</v>
-      </c>
-      <c r="E612" s="2" t="inlineStr"/>
+        <v>527150</v>
+      </c>
+      <c r="E612" s="4" t="n">
+        <v>0.9698</v>
+      </c>
       <c r="F612" s="3" t="n">
-        <v>36.71</v>
+        <v>45.64</v>
       </c>
       <c r="G612" s="2" t="inlineStr"/>
       <c r="H612" s="2" t="inlineStr"/>
       <c r="I612" s="2" t="inlineStr"/>
-      <c r="J612" s="2" t="inlineStr"/>
+      <c r="J612" s="4" t="n">
+        <v>0.6453</v>
+      </c>
       <c r="K612" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L612" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M612" s="2" t="inlineStr"/>
@@ -26852,7 +26852,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>27.05.2026 14:30</t>
+          <t>27.05.2026 15:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 27.05.2026 16:30 | 611 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-27.xlsx
+++ b/data/bist_screener_2026-05-27.xlsx
@@ -25942,58 +25942,56 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>36.38</v>
+        <v>70.25</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.0022</v>
+        <v>0.09939999999999999</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>23850000</v>
+        <v>42550</v>
       </c>
       <c r="E588" s="4" t="n">
-        <v>0.2667</v>
+        <v>0.58</v>
       </c>
       <c r="F588" s="3" t="n">
-        <v>68.22</v>
+        <v>44.2</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
       <c r="I588" s="2" t="inlineStr"/>
-      <c r="J588" s="2" t="inlineStr"/>
+      <c r="J588" s="4" t="n">
+        <v>0.4928</v>
+      </c>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L588" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L588" s="2" t="inlineStr"/>
       <c r="M588" s="2" t="inlineStr"/>
     </row>
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>17.67</v>
+        <v>170.1</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0172</v>
+        <v>-0.023</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>21980000</v>
+        <v>6070000</v>
       </c>
       <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>36.71</v>
+        <v>38.2</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -26001,12 +25999,12 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26014,34 +26012,40 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>74.05</v>
+        <v>129.6</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.0886</v>
+        <v>-0.0077</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>25520000</v>
-      </c>
-      <c r="E590" s="2" t="inlineStr"/>
+        <v>879570</v>
+      </c>
+      <c r="E590" s="4" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F590" s="3" t="n">
-        <v>67.18000000000001</v>
+        <v>41.79</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
-      <c r="I590" s="2" t="inlineStr"/>
-      <c r="J590" s="2" t="inlineStr"/>
+      <c r="I590" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J590" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26049,93 +26053,83 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>40.96</v>
+        <v>80.37</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0039</v>
+        <v>-0.0042</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>4380000</v>
+        <v>11050000</v>
       </c>
       <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>50.43</v>
+        <v>49.24</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
       <c r="I591" s="6" t="inlineStr"/>
       <c r="J591" s="6" t="inlineStr"/>
-      <c r="K591" s="6" t="inlineStr">
-        <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L591" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
-        </is>
-      </c>
+      <c r="K591" s="6" t="inlineStr"/>
+      <c r="L591" s="6" t="inlineStr"/>
       <c r="M591" s="6" t="inlineStr"/>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>12</v>
+        <v>191.9</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.0345</v>
+        <v>-0.0174</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>498860</v>
-      </c>
-      <c r="E592" s="4" t="n">
-        <v>0.95</v>
-      </c>
+        <v>5800000</v>
+      </c>
+      <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>69.81999999999999</v>
+        <v>55.81</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
-      <c r="I592" s="4" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J592" s="4" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I592" s="2" t="inlineStr"/>
+      <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L592" s="2" t="inlineStr"/>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+        </is>
+      </c>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>2.6</v>
+        <v>6.12</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0189</v>
+        <v>0.009899999999999999</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>94430000</v>
+        <v>8660000</v>
       </c>
       <c r="E593" s="6" t="inlineStr"/>
       <c r="F593" s="7" t="n">
-        <v>42.83</v>
+        <v>54.27</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
@@ -26146,52 +26140,40 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L593" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+      <c r="L593" s="6" t="inlineStr"/>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>34.72</v>
+        <v>17.67</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.0012</v>
+        <v>-0.0172</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>4640000</v>
-      </c>
-      <c r="E594" s="4" t="n">
-        <v>0.3528</v>
-      </c>
+        <v>21980000</v>
+      </c>
+      <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>46.16</v>
-      </c>
-      <c r="G594" s="3" t="n">
-        <v>13.72</v>
-      </c>
+        <v>36.71</v>
+      </c>
+      <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="4" t="n">
-        <v>0.1029</v>
-      </c>
-      <c r="J594" s="4" t="n">
-        <v>-1.4864</v>
-      </c>
+      <c r="I594" s="2" t="inlineStr"/>
+      <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26199,40 +26181,34 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>5.87</v>
+        <v>39.6</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.0731</v>
+        <v>-0.0365</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>18100000</v>
-      </c>
-      <c r="E595" s="8" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>11700000</v>
+      </c>
+      <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="7" t="n">
-        <v>49.01</v>
+        <v>59.52</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
-      <c r="I595" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J595" s="8" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I595" s="6" t="inlineStr"/>
+      <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26240,29 +26216,35 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>77</v>
+        <v>12</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0158</v>
+        <v>0.0345</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>137290</v>
-      </c>
-      <c r="E596" s="2" t="inlineStr"/>
+        <v>498860</v>
+      </c>
+      <c r="E596" s="4" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F596" s="3" t="n">
-        <v>28.48</v>
+        <v>69.81999999999999</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="2" t="inlineStr"/>
-      <c r="J596" s="2" t="inlineStr"/>
+      <c r="I596" s="4" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J596" s="4" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr"/>
@@ -26271,38 +26253,34 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>67.15000000000001</v>
+        <v>16.49</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0121</v>
+        <v>0.005500000000000001</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>562280</v>
-      </c>
-      <c r="E597" s="8" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>28260000</v>
+      </c>
+      <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>54.15</v>
+        <v>48.12</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
       <c r="I597" s="6" t="inlineStr"/>
-      <c r="J597" s="8" t="n">
-        <v>0.1431</v>
-      </c>
+      <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26310,34 +26288,38 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>39.6</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0365</v>
+        <v>0.0121</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>11700000</v>
-      </c>
-      <c r="E598" s="2" t="inlineStr"/>
+        <v>562280</v>
+      </c>
+      <c r="E598" s="4" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F598" s="3" t="n">
-        <v>59.52</v>
+        <v>54.15</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
       <c r="I598" s="2" t="inlineStr"/>
-      <c r="J598" s="2" t="inlineStr"/>
+      <c r="J598" s="4" t="n">
+        <v>0.1431</v>
+      </c>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26345,21 +26327,21 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>6.12</v>
+        <v>13.92</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.009899999999999999</v>
+        <v>-0.0029</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>8660000</v>
+        <v>19750000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>54.27</v>
+        <v>50.28</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26367,43 +26349,43 @@
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L599" s="6" t="inlineStr"/>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L599" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>EKDMR</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>191.9</v>
+        <v>59.85</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>-0.0174</v>
-      </c>
-      <c r="D600" s="5" t="n">
-        <v>5800000</v>
-      </c>
+        <v>0.0992</v>
+      </c>
+      <c r="D600" s="2" t="inlineStr"/>
       <c r="E600" s="2" t="inlineStr"/>
-      <c r="F600" s="3" t="n">
-        <v>55.81</v>
-      </c>
+      <c r="F600" s="2" t="inlineStr"/>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
       <c r="I600" s="2" t="inlineStr"/>
       <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Enerji-dışı mineraller</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST HALKA ARZ, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26411,104 +26393,106 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>245</v>
+        <v>2.4</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.0298</v>
+        <v>0</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>9560</v>
+        <v>16980000</v>
       </c>
       <c r="E601" s="8" t="n">
-        <v>0.2578</v>
+        <v>1</v>
       </c>
       <c r="F601" s="7" t="n">
-        <v>50.37</v>
+        <v>39.22</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="6" t="inlineStr"/>
-      <c r="J601" s="6" t="inlineStr"/>
+      <c r="I601" s="8" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J601" s="8" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L601" s="6" t="inlineStr"/>
+          <t>Dağıtım servisleri</t>
+        </is>
+      </c>
+      <c r="L601" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+        </is>
+      </c>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>EKDMR</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>59.85</v>
+        <v>77</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.0992</v>
-      </c>
-      <c r="D602" s="2" t="inlineStr"/>
+        <v>0.0158</v>
+      </c>
+      <c r="D602" s="5" t="n">
+        <v>137290</v>
+      </c>
       <c r="E602" s="2" t="inlineStr"/>
-      <c r="F602" s="2" t="inlineStr"/>
+      <c r="F602" s="3" t="n">
+        <v>28.48</v>
+      </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
       <c r="I602" s="2" t="inlineStr"/>
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
-        </is>
-      </c>
-      <c r="L602" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST HALKA ARZ, BIST YILDIZ</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L602" s="2" t="inlineStr"/>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>129.6</v>
+        <v>32.18</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.0077</v>
+        <v>0.0255</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>879570</v>
-      </c>
-      <c r="E603" s="8" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>17120000</v>
+      </c>
+      <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>41.79</v>
+        <v>65.51000000000001</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="8" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J603" s="8" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I603" s="6" t="inlineStr"/>
+      <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26516,21 +26500,21 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>32.18</v>
+        <v>2.6</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0.0255</v>
+        <v>-0.0189</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>17120000</v>
+        <v>94430000</v>
       </c>
       <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>65.51000000000001</v>
+        <v>42.83</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26538,12 +26522,12 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26551,40 +26535,42 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>2.4</v>
+        <v>34.72</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0</v>
+        <v>-0.0012</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>16980000</v>
+        <v>4640000</v>
       </c>
       <c r="E605" s="8" t="n">
-        <v>1</v>
+        <v>0.3528</v>
       </c>
       <c r="F605" s="7" t="n">
-        <v>39.22</v>
-      </c>
-      <c r="G605" s="6" t="inlineStr"/>
+        <v>46.16</v>
+      </c>
+      <c r="G605" s="7" t="n">
+        <v>13.72</v>
+      </c>
       <c r="H605" s="6" t="inlineStr"/>
       <c r="I605" s="8" t="n">
-        <v>-191.6342</v>
+        <v>0.1029</v>
       </c>
       <c r="J605" s="8" t="n">
-        <v>-0.8093</v>
+        <v>-1.4864</v>
       </c>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26592,21 +26578,23 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>13.92</v>
+        <v>36.38</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.0029</v>
+        <v>0.0022</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>19750000</v>
-      </c>
-      <c r="E606" s="2" t="inlineStr"/>
+        <v>23850000</v>
+      </c>
+      <c r="E606" s="4" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F606" s="3" t="n">
-        <v>50.28</v>
+        <v>68.22</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
@@ -26614,12 +26602,12 @@
       <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26627,21 +26615,21 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>170.1</v>
+        <v>40.96</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.023</v>
+        <v>0.0039</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>6070000</v>
+        <v>4380000</v>
       </c>
       <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>38.2</v>
+        <v>50.43</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26649,12 +26637,12 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26662,83 +26650,99 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>70.25</v>
+        <v>74.05</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>0.09939999999999999</v>
+        <v>-0.0886</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>42550</v>
-      </c>
-      <c r="E608" s="4" t="n">
-        <v>0.58</v>
-      </c>
+        <v>25520000</v>
+      </c>
+      <c r="E608" s="2" t="inlineStr"/>
       <c r="F608" s="3" t="n">
-        <v>44.2</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
       <c r="I608" s="2" t="inlineStr"/>
-      <c r="J608" s="4" t="n">
-        <v>0.4928</v>
-      </c>
+      <c r="J608" s="2" t="inlineStr"/>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L608" s="2" t="inlineStr"/>
+          <t>Elektronik teknoloji</t>
+        </is>
+      </c>
+      <c r="L608" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+        </is>
+      </c>
       <c r="M608" s="2" t="inlineStr"/>
     </row>
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>80.37</v>
+        <v>5.87</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>-0.0042</v>
+        <v>0.0731</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>11050000</v>
-      </c>
-      <c r="E609" s="6" t="inlineStr"/>
+        <v>18100000</v>
+      </c>
+      <c r="E609" s="8" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F609" s="7" t="n">
-        <v>49.24</v>
+        <v>49.01</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
-      <c r="I609" s="6" t="inlineStr"/>
-      <c r="J609" s="6" t="inlineStr"/>
-      <c r="K609" s="6" t="inlineStr"/>
-      <c r="L609" s="6" t="inlineStr"/>
+      <c r="I609" s="8" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J609" s="8" t="n">
+        <v>-4.2562</v>
+      </c>
+      <c r="K609" s="6" t="inlineStr">
+        <is>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L609" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M609" s="6" t="inlineStr"/>
     </row>
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>16.3</v>
+        <v>245</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>-0.0151</v>
+        <v>0.0298</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>30420000</v>
-      </c>
-      <c r="E610" s="2" t="inlineStr"/>
+        <v>9560</v>
+      </c>
+      <c r="E610" s="4" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F610" s="3" t="n">
-        <v>45.98</v>
+        <v>50.37</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
@@ -26746,47 +26750,47 @@
       <c r="J610" s="2" t="inlineStr"/>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L610" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L610" s="2" t="inlineStr"/>
       <c r="M610" s="2" t="inlineStr"/>
     </row>
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>16.49</v>
+        <v>25.7</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>0.005500000000000001</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>28260000</v>
-      </c>
-      <c r="E611" s="6" t="inlineStr"/>
+        <v>527150</v>
+      </c>
+      <c r="E611" s="8" t="n">
+        <v>0.9698</v>
+      </c>
       <c r="F611" s="7" t="n">
-        <v>48.12</v>
+        <v>45.64</v>
       </c>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
       <c r="I611" s="6" t="inlineStr"/>
-      <c r="J611" s="6" t="inlineStr"/>
+      <c r="J611" s="8" t="n">
+        <v>0.6453</v>
+      </c>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L611" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M611" s="6" t="inlineStr"/>
@@ -26794,38 +26798,34 @@
     <row r="612">
       <c r="A612" s="2" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B612" s="3" t="n">
-        <v>25.7</v>
+        <v>16.3</v>
       </c>
       <c r="C612" s="4" t="n">
-        <v>-0.006999999999999999</v>
+        <v>-0.0151</v>
       </c>
       <c r="D612" s="5" t="n">
-        <v>527150</v>
-      </c>
-      <c r="E612" s="4" t="n">
-        <v>0.9698</v>
-      </c>
+        <v>30420000</v>
+      </c>
+      <c r="E612" s="2" t="inlineStr"/>
       <c r="F612" s="3" t="n">
-        <v>45.64</v>
+        <v>45.98</v>
       </c>
       <c r="G612" s="2" t="inlineStr"/>
       <c r="H612" s="2" t="inlineStr"/>
       <c r="I612" s="2" t="inlineStr"/>
-      <c r="J612" s="4" t="n">
-        <v>0.6453</v>
-      </c>
+      <c r="J612" s="2" t="inlineStr"/>
       <c r="K612" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L612" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M612" s="2" t="inlineStr"/>
@@ -26852,7 +26852,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>27.05.2026 15:30</t>
+          <t>27.05.2026 16:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 27.05.2026 18:10 | 611 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-27.xlsx
+++ b/data/bist_screener_2026-05-27.xlsx
@@ -25942,56 +25942,58 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>70.25</v>
+        <v>16.49</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.09939999999999999</v>
+        <v>0.005500000000000001</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>42550</v>
-      </c>
-      <c r="E588" s="4" t="n">
-        <v>0.58</v>
-      </c>
+        <v>28260000</v>
+      </c>
+      <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>44.2</v>
+        <v>48.12</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
       <c r="I588" s="2" t="inlineStr"/>
-      <c r="J588" s="4" t="n">
-        <v>0.4928</v>
-      </c>
+      <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L588" s="2" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L588" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M588" s="2" t="inlineStr"/>
     </row>
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>170.1</v>
+        <v>245</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.023</v>
+        <v>0.0298</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>6070000</v>
-      </c>
-      <c r="E589" s="6" t="inlineStr"/>
+        <v>9560</v>
+      </c>
+      <c r="E589" s="8" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F589" s="7" t="n">
-        <v>38.2</v>
+        <v>50.37</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -25999,53 +26001,49 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L589" s="6" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L589" s="6" t="inlineStr"/>
       <c r="M589" s="6" t="inlineStr"/>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>129.6</v>
+        <v>2.4</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.0077</v>
+        <v>0</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>879570</v>
+        <v>16980000</v>
       </c>
       <c r="E590" s="4" t="n">
-        <v>0.1071</v>
+        <v>1</v>
       </c>
       <c r="F590" s="3" t="n">
-        <v>41.79</v>
+        <v>39.22</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
       <c r="I590" s="4" t="n">
-        <v>-3.6635</v>
+        <v>-191.6342</v>
       </c>
       <c r="J590" s="4" t="n">
-        <v>-0.4897</v>
+        <v>-0.8093</v>
       </c>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26053,48 +26051,56 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>80.37</v>
+        <v>39.6</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>-0.0042</v>
+        <v>-0.0365</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>11050000</v>
+        <v>11700000</v>
       </c>
       <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>49.24</v>
+        <v>59.52</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
       <c r="I591" s="6" t="inlineStr"/>
       <c r="J591" s="6" t="inlineStr"/>
-      <c r="K591" s="6" t="inlineStr"/>
-      <c r="L591" s="6" t="inlineStr"/>
+      <c r="K591" s="6" t="inlineStr">
+        <is>
+          <t>Üretici imalatı</t>
+        </is>
+      </c>
+      <c r="L591" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+        </is>
+      </c>
       <c r="M591" s="6" t="inlineStr"/>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>191.9</v>
+        <v>40.96</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.0174</v>
+        <v>0.0039</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>5800000</v>
+        <v>4380000</v>
       </c>
       <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>55.81</v>
+        <v>50.43</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
@@ -26102,12 +26108,12 @@
       <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26115,21 +26121,21 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>6.12</v>
+        <v>170.1</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0.009899999999999999</v>
+        <v>-0.023</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>8660000</v>
+        <v>6070000</v>
       </c>
       <c r="E593" s="6" t="inlineStr"/>
       <c r="F593" s="7" t="n">
-        <v>54.27</v>
+        <v>38.2</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
@@ -26137,30 +26143,34 @@
       <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L593" s="6" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L593" s="6" t="inlineStr">
+        <is>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+        </is>
+      </c>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>17.67</v>
+        <v>32.18</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.0172</v>
+        <v>0.0255</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>21980000</v>
+        <v>17120000</v>
       </c>
       <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>36.71</v>
+        <v>65.51000000000001</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
@@ -26168,12 +26178,12 @@
       <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26181,34 +26191,40 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>39.6</v>
+        <v>5.87</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.0365</v>
+        <v>0.0731</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>11700000</v>
-      </c>
-      <c r="E595" s="6" t="inlineStr"/>
+        <v>18100000</v>
+      </c>
+      <c r="E595" s="8" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F595" s="7" t="n">
-        <v>59.52</v>
+        <v>49.01</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
-      <c r="I595" s="6" t="inlineStr"/>
-      <c r="J595" s="6" t="inlineStr"/>
+      <c r="I595" s="8" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J595" s="8" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26216,110 +26232,96 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>12</v>
+        <v>16.3</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0345</v>
+        <v>-0.0151</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>498860</v>
-      </c>
-      <c r="E596" s="4" t="n">
-        <v>0.95</v>
-      </c>
+        <v>30420000</v>
+      </c>
+      <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>69.81999999999999</v>
+        <v>45.98</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="4" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J596" s="4" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I596" s="2" t="inlineStr"/>
+      <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L596" s="2" t="inlineStr"/>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L596" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+        </is>
+      </c>
       <c r="M596" s="2" t="inlineStr"/>
     </row>
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>16.49</v>
+        <v>80.37</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.005500000000000001</v>
+        <v>-0.0042</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>28260000</v>
+        <v>11050000</v>
       </c>
       <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>48.12</v>
+        <v>49.24</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
       <c r="I597" s="6" t="inlineStr"/>
       <c r="J597" s="6" t="inlineStr"/>
-      <c r="K597" s="6" t="inlineStr">
-        <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L597" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+      <c r="K597" s="6" t="inlineStr"/>
+      <c r="L597" s="6" t="inlineStr"/>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>67.15000000000001</v>
+        <v>191.9</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>0.0121</v>
+        <v>-0.0174</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>562280</v>
-      </c>
-      <c r="E598" s="4" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>5800000</v>
+      </c>
+      <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>54.15</v>
+        <v>55.81</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
       <c r="I598" s="2" t="inlineStr"/>
-      <c r="J598" s="4" t="n">
-        <v>0.1431</v>
-      </c>
+      <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26327,21 +26329,23 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>13.92</v>
+        <v>36.38</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0029</v>
+        <v>0.0022</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>19750000</v>
-      </c>
-      <c r="E599" s="6" t="inlineStr"/>
+        <v>23850000</v>
+      </c>
+      <c r="E599" s="8" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F599" s="7" t="n">
-        <v>50.28</v>
+        <v>68.22</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26349,12 +26353,12 @@
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26362,30 +26366,38 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>EKDMR</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>59.85</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.0992</v>
-      </c>
-      <c r="D600" s="2" t="inlineStr"/>
-      <c r="E600" s="2" t="inlineStr"/>
-      <c r="F600" s="2" t="inlineStr"/>
+        <v>0.0121</v>
+      </c>
+      <c r="D600" s="5" t="n">
+        <v>562280</v>
+      </c>
+      <c r="E600" s="4" t="n">
+        <v>0.3695000000000001</v>
+      </c>
+      <c r="F600" s="3" t="n">
+        <v>54.15</v>
+      </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
       <c r="I600" s="2" t="inlineStr"/>
-      <c r="J600" s="2" t="inlineStr"/>
+      <c r="J600" s="4" t="n">
+        <v>0.1431</v>
+      </c>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST HALKA ARZ, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26393,70 +26405,70 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>2.4</v>
+        <v>70.25</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0</v>
+        <v>0.09939999999999999</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>16980000</v>
+        <v>42550</v>
       </c>
       <c r="E601" s="8" t="n">
-        <v>1</v>
+        <v>0.58</v>
       </c>
       <c r="F601" s="7" t="n">
-        <v>39.22</v>
+        <v>44.2</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
+      <c r="I601" s="6" t="inlineStr"/>
       <c r="J601" s="8" t="n">
-        <v>-0.8093</v>
+        <v>0.4928</v>
       </c>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
-        </is>
-      </c>
-      <c r="L601" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L601" s="6" t="inlineStr"/>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>77</v>
+        <v>12</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.0158</v>
+        <v>0.0345</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>137290</v>
-      </c>
-      <c r="E602" s="2" t="inlineStr"/>
+        <v>498860</v>
+      </c>
+      <c r="E602" s="4" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F602" s="3" t="n">
-        <v>28.48</v>
+        <v>69.81999999999999</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
-      <c r="I602" s="2" t="inlineStr"/>
-      <c r="J602" s="2" t="inlineStr"/>
+      <c r="I602" s="4" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J602" s="4" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr"/>
@@ -26465,21 +26477,21 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>32.18</v>
+        <v>2.6</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0255</v>
+        <v>-0.0189</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>17120000</v>
+        <v>94430000</v>
       </c>
       <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>65.51000000000001</v>
+        <v>42.83</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
@@ -26487,12 +26499,12 @@
       <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26500,21 +26512,21 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>2.6</v>
+        <v>77</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0189</v>
+        <v>0.0158</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>94430000</v>
+        <v>137290</v>
       </c>
       <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>42.83</v>
+        <v>28.48</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26525,43 +26537,35 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L604" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+      <c r="L604" s="2" t="inlineStr"/>
       <c r="M604" s="2" t="inlineStr"/>
     </row>
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>34.72</v>
+        <v>25.7</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.0012</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>4640000</v>
+        <v>527150</v>
       </c>
       <c r="E605" s="8" t="n">
-        <v>0.3528</v>
+        <v>0.9698</v>
       </c>
       <c r="F605" s="7" t="n">
-        <v>46.16</v>
-      </c>
-      <c r="G605" s="7" t="n">
-        <v>13.72</v>
-      </c>
+        <v>45.64</v>
+      </c>
+      <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
-      <c r="I605" s="8" t="n">
-        <v>0.1029</v>
-      </c>
+      <c r="I605" s="6" t="inlineStr"/>
       <c r="J605" s="8" t="n">
-        <v>-1.4864</v>
+        <v>0.6453</v>
       </c>
       <c r="K605" s="6" t="inlineStr">
         <is>
@@ -26570,7 +26574,7 @@
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26578,36 +26582,42 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>36.38</v>
+        <v>34.72</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.0022</v>
+        <v>-0.0012</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>23850000</v>
+        <v>4640000</v>
       </c>
       <c r="E606" s="4" t="n">
-        <v>0.2667</v>
+        <v>0.3528</v>
       </c>
       <c r="F606" s="3" t="n">
-        <v>68.22</v>
-      </c>
-      <c r="G606" s="2" t="inlineStr"/>
+        <v>46.16</v>
+      </c>
+      <c r="G606" s="3" t="n">
+        <v>13.72</v>
+      </c>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="2" t="inlineStr"/>
-      <c r="J606" s="2" t="inlineStr"/>
+      <c r="I606" s="4" t="n">
+        <v>0.1029</v>
+      </c>
+      <c r="J606" s="4" t="n">
+        <v>-1.4864</v>
+      </c>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26615,21 +26625,21 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>40.96</v>
+        <v>6.12</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>0.0039</v>
+        <v>0.009899999999999999</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>4380000</v>
+        <v>8660000</v>
       </c>
       <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>50.43</v>
+        <v>54.27</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26637,34 +26647,30 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L607" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L607" s="6" t="inlineStr"/>
       <c r="M607" s="6" t="inlineStr"/>
     </row>
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>74.05</v>
+        <v>17.67</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>-0.0886</v>
+        <v>-0.0172</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>25520000</v>
+        <v>21980000</v>
       </c>
       <c r="E608" s="2" t="inlineStr"/>
       <c r="F608" s="3" t="n">
-        <v>67.18000000000001</v>
+        <v>36.71</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
@@ -26672,12 +26678,12 @@
       <c r="J608" s="2" t="inlineStr"/>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L608" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M608" s="2" t="inlineStr"/>
@@ -26685,40 +26691,30 @@
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>EKDMR</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>5.87</v>
+        <v>59.85</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>0.0731</v>
-      </c>
-      <c r="D609" s="9" t="n">
-        <v>18100000</v>
-      </c>
-      <c r="E609" s="8" t="n">
-        <v>0.1672</v>
-      </c>
-      <c r="F609" s="7" t="n">
-        <v>49.01</v>
-      </c>
+        <v>0.0992</v>
+      </c>
+      <c r="D609" s="6" t="inlineStr"/>
+      <c r="E609" s="6" t="inlineStr"/>
+      <c r="F609" s="6" t="inlineStr"/>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
-      <c r="I609" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J609" s="8" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I609" s="6" t="inlineStr"/>
+      <c r="J609" s="6" t="inlineStr"/>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Enerji-dışı mineraller</t>
         </is>
       </c>
       <c r="L609" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST HALKA ARZ, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M609" s="6" t="inlineStr"/>
@@ -26726,23 +26722,21 @@
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>245</v>
+        <v>13.92</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>0.0298</v>
+        <v>-0.0029</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>9560</v>
-      </c>
-      <c r="E610" s="4" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>19750000</v>
+      </c>
+      <c r="E610" s="2" t="inlineStr"/>
       <c r="F610" s="3" t="n">
-        <v>50.37</v>
+        <v>50.28</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
@@ -26753,44 +26747,44 @@
           <t>İşlenebilen endüstriler</t>
         </is>
       </c>
-      <c r="L610" s="2" t="inlineStr"/>
+      <c r="L610" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M610" s="2" t="inlineStr"/>
     </row>
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>25.7</v>
+        <v>74.05</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>-0.006999999999999999</v>
+        <v>-0.0886</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>527150</v>
-      </c>
-      <c r="E611" s="8" t="n">
-        <v>0.9698</v>
-      </c>
+        <v>25520000</v>
+      </c>
+      <c r="E611" s="6" t="inlineStr"/>
       <c r="F611" s="7" t="n">
-        <v>45.64</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
       <c r="I611" s="6" t="inlineStr"/>
-      <c r="J611" s="8" t="n">
-        <v>0.6453</v>
-      </c>
+      <c r="J611" s="6" t="inlineStr"/>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L611" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M611" s="6" t="inlineStr"/>
@@ -26798,34 +26792,40 @@
     <row r="612">
       <c r="A612" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B612" s="3" t="n">
-        <v>16.3</v>
+        <v>129.6</v>
       </c>
       <c r="C612" s="4" t="n">
-        <v>-0.0151</v>
+        <v>-0.0077</v>
       </c>
       <c r="D612" s="5" t="n">
-        <v>30420000</v>
-      </c>
-      <c r="E612" s="2" t="inlineStr"/>
+        <v>879570</v>
+      </c>
+      <c r="E612" s="4" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F612" s="3" t="n">
-        <v>45.98</v>
+        <v>41.79</v>
       </c>
       <c r="G612" s="2" t="inlineStr"/>
       <c r="H612" s="2" t="inlineStr"/>
-      <c r="I612" s="2" t="inlineStr"/>
-      <c r="J612" s="2" t="inlineStr"/>
+      <c r="I612" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J612" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K612" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L612" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M612" s="2" t="inlineStr"/>
@@ -26852,7 +26852,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>27.05.2026 16:30</t>
+          <t>27.05.2026 18:10</t>
         </is>
       </c>
     </row>

</xml_diff>